<commit_message>
fix: swipe filter breakoutboard VCC to main connector side
</commit_message>
<xml_diff>
--- a/ODB_V3/Hardware/Kicad/STM32F412ZGT6_Interfaces.xlsx
+++ b/ODB_V3/Hardware/Kicad/STM32F412ZGT6_Interfaces.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gagno\OneDrive\Documents\Ulaval\GAUL\ODB2\Ordinateur-de-bord\ODB_V3\Hardware\Kicad\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gagno\OneDrive\Documents\ULaval\GAUL\ODB2\Ordinateur-de-bord\ODB_V3\Hardware\Kicad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E424EB1-66AF-4A29-AF6F-A42E181CC79D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0191D53-32D2-4AB7-B999-89BFA3C6C21B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18780" yWindow="0" windowWidth="32925" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2490" yWindow="3015" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="192">
   <si>
     <t>Interface</t>
   </si>
@@ -585,9 +585,6 @@
   </si>
   <si>
     <t>UART6</t>
-  </si>
-  <si>
-    <t>I2C1</t>
   </si>
   <si>
     <t>I2C2</t>
@@ -967,31 +964,43 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1002,18 +1011,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1418,16 +1415,16 @@
       </c>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B3" s="54" t="s">
+      <c r="B3" s="43" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="56">
+      <c r="C3" s="50">
         <v>1</v>
       </c>
-      <c r="D3" s="48" t="s">
+      <c r="D3" s="47" t="s">
         <v>90</v>
       </c>
-      <c r="E3" s="48" t="s">
+      <c r="E3" s="47" t="s">
         <v>70</v>
       </c>
       <c r="F3" s="15" t="s">
@@ -1442,7 +1439,7 @@
       <c r="I3" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="K3" s="54" t="s">
+      <c r="K3" s="43" t="s">
         <v>94</v>
       </c>
       <c r="L3" s="22" t="s">
@@ -1450,10 +1447,10 @@
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B4" s="54"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="49"/>
-      <c r="E4" s="49"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="51"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
       <c r="F4" s="2" t="s">
         <v>2</v>
       </c>
@@ -1466,16 +1463,16 @@
       <c r="I4" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="K4" s="54"/>
+      <c r="K4" s="43"/>
       <c r="L4" s="23" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="54"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="49"/>
-      <c r="E5" s="49"/>
+      <c r="B5" s="43"/>
+      <c r="C5" s="51"/>
+      <c r="D5" s="48"/>
+      <c r="E5" s="48"/>
       <c r="F5" s="2" t="s">
         <v>3</v>
       </c>
@@ -1496,10 +1493,10 @@
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B6" s="54"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="49"/>
+      <c r="B6" s="43"/>
+      <c r="C6" s="51"/>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
       <c r="F6" s="2" t="s">
         <v>64</v>
       </c>
@@ -1512,7 +1509,7 @@
       <c r="I6" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="K6" s="54" t="s">
+      <c r="K6" s="43" t="s">
         <v>101</v>
       </c>
       <c r="L6" s="22" t="s">
@@ -1520,14 +1517,14 @@
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B7" s="54"/>
-      <c r="C7" s="56">
+      <c r="B7" s="43"/>
+      <c r="C7" s="50">
         <v>2</v>
       </c>
-      <c r="D7" s="48" t="s">
+      <c r="D7" s="47" t="s">
         <v>91</v>
       </c>
-      <c r="E7" s="48" t="s">
+      <c r="E7" s="47" t="s">
         <v>71</v>
       </c>
       <c r="F7" s="15" t="s">
@@ -1542,16 +1539,16 @@
       <c r="I7" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="K7" s="54"/>
+      <c r="K7" s="43"/>
       <c r="L7" s="23" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B8" s="54"/>
-      <c r="C8" s="44"/>
-      <c r="D8" s="49"/>
-      <c r="E8" s="49"/>
+      <c r="B8" s="43"/>
+      <c r="C8" s="51"/>
+      <c r="D8" s="48"/>
+      <c r="E8" s="48"/>
       <c r="F8" s="2" t="s">
         <v>2</v>
       </c>
@@ -1572,10 +1569,10 @@
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B9" s="54"/>
-      <c r="C9" s="44"/>
-      <c r="D9" s="49"/>
-      <c r="E9" s="49"/>
+      <c r="B9" s="43"/>
+      <c r="C9" s="51"/>
+      <c r="D9" s="48"/>
+      <c r="E9" s="48"/>
       <c r="F9" s="2" t="s">
         <v>3</v>
       </c>
@@ -1596,10 +1593,10 @@
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B10" s="54"/>
-      <c r="C10" s="55"/>
-      <c r="D10" s="50"/>
-      <c r="E10" s="50"/>
+      <c r="B10" s="43"/>
+      <c r="C10" s="52"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="49"/>
       <c r="F10" s="9" t="s">
         <v>64</v>
       </c>
@@ -1612,19 +1609,19 @@
       <c r="I10" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="K10" s="42" t="s">
+      <c r="K10" s="44" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="54"/>
-      <c r="C11" s="56">
+      <c r="B11" s="43"/>
+      <c r="C11" s="50">
         <v>3</v>
       </c>
-      <c r="D11" s="48" t="s">
+      <c r="D11" s="47" t="s">
         <v>91</v>
       </c>
-      <c r="E11" s="48" t="s">
+      <c r="E11" s="47" t="s">
         <v>71</v>
       </c>
       <c r="F11" s="15" t="s">
@@ -1639,13 +1636,13 @@
       <c r="I11" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="K11" s="43"/>
+      <c r="K11" s="45"/>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B12" s="54"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="49"/>
-      <c r="E12" s="49"/>
+      <c r="B12" s="43"/>
+      <c r="C12" s="51"/>
+      <c r="D12" s="48"/>
+      <c r="E12" s="48"/>
       <c r="F12" s="2" t="s">
         <v>2</v>
       </c>
@@ -1658,13 +1655,13 @@
       <c r="I12" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="K12" s="43"/>
+      <c r="K12" s="45"/>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B13" s="54"/>
-      <c r="C13" s="44"/>
-      <c r="D13" s="49"/>
-      <c r="E13" s="49"/>
+      <c r="B13" s="43"/>
+      <c r="C13" s="51"/>
+      <c r="D13" s="48"/>
+      <c r="E13" s="48"/>
       <c r="F13" s="2" t="s">
         <v>3</v>
       </c>
@@ -1677,13 +1674,13 @@
       <c r="I13" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="K13" s="43"/>
+      <c r="K13" s="45"/>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B14" s="54"/>
-      <c r="C14" s="55"/>
-      <c r="D14" s="50"/>
-      <c r="E14" s="50"/>
+      <c r="B14" s="43"/>
+      <c r="C14" s="52"/>
+      <c r="D14" s="49"/>
+      <c r="E14" s="49"/>
       <c r="F14" s="9" t="s">
         <v>64</v>
       </c>
@@ -1696,17 +1693,17 @@
       <c r="I14" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="K14" s="43"/>
+      <c r="K14" s="45"/>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B15" s="54"/>
-      <c r="C15" s="56">
+      <c r="B15" s="43"/>
+      <c r="C15" s="50">
         <v>4</v>
       </c>
-      <c r="D15" s="48" t="s">
+      <c r="D15" s="47" t="s">
         <v>90</v>
       </c>
-      <c r="E15" s="48" t="s">
+      <c r="E15" s="47" t="s">
         <v>70</v>
       </c>
       <c r="F15" s="15" t="s">
@@ -1721,13 +1718,13 @@
       <c r="I15" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="K15" s="43"/>
+      <c r="K15" s="45"/>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B16" s="54"/>
-      <c r="C16" s="44"/>
-      <c r="D16" s="49"/>
-      <c r="E16" s="49"/>
+      <c r="B16" s="43"/>
+      <c r="C16" s="51"/>
+      <c r="D16" s="48"/>
+      <c r="E16" s="48"/>
       <c r="F16" s="2" t="s">
         <v>2</v>
       </c>
@@ -1740,13 +1737,13 @@
       <c r="I16" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="K16" s="43"/>
+      <c r="K16" s="45"/>
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B17" s="54"/>
-      <c r="C17" s="44"/>
-      <c r="D17" s="49"/>
-      <c r="E17" s="49"/>
+      <c r="B17" s="43"/>
+      <c r="C17" s="51"/>
+      <c r="D17" s="48"/>
+      <c r="E17" s="48"/>
       <c r="F17" s="2" t="s">
         <v>3</v>
       </c>
@@ -1759,13 +1756,13 @@
       <c r="I17" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="K17" s="43"/>
+      <c r="K17" s="45"/>
     </row>
     <row r="18" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B18" s="54"/>
-      <c r="C18" s="55"/>
-      <c r="D18" s="50"/>
-      <c r="E18" s="50"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="52"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="49"/>
       <c r="F18" s="9" t="s">
         <v>64</v>
       </c>
@@ -1778,17 +1775,17 @@
       <c r="I18" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="K18" s="43"/>
+      <c r="K18" s="45"/>
     </row>
     <row r="19" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B19" s="54"/>
-      <c r="C19" s="56">
+      <c r="B19" s="43"/>
+      <c r="C19" s="50">
         <v>5</v>
       </c>
-      <c r="D19" s="48" t="s">
+      <c r="D19" s="47" t="s">
         <v>90</v>
       </c>
-      <c r="E19" s="48" t="s">
+      <c r="E19" s="47" t="s">
         <v>70</v>
       </c>
       <c r="F19" s="15" t="s">
@@ -1803,13 +1800,13 @@
       <c r="I19" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="K19" s="43"/>
+      <c r="K19" s="45"/>
     </row>
     <row r="20" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B20" s="54"/>
-      <c r="C20" s="44"/>
-      <c r="D20" s="49"/>
-      <c r="E20" s="49"/>
+      <c r="B20" s="43"/>
+      <c r="C20" s="51"/>
+      <c r="D20" s="48"/>
+      <c r="E20" s="48"/>
       <c r="F20" s="2" t="s">
         <v>2</v>
       </c>
@@ -1822,13 +1819,13 @@
       <c r="I20" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="K20" s="43"/>
+      <c r="K20" s="45"/>
     </row>
     <row r="21" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B21" s="54"/>
-      <c r="C21" s="44"/>
-      <c r="D21" s="49"/>
-      <c r="E21" s="49"/>
+      <c r="B21" s="43"/>
+      <c r="C21" s="51"/>
+      <c r="D21" s="48"/>
+      <c r="E21" s="48"/>
       <c r="F21" s="2" t="s">
         <v>3</v>
       </c>
@@ -1841,13 +1838,13 @@
       <c r="I21" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="K21" s="43"/>
+      <c r="K21" s="45"/>
     </row>
     <row r="22" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B22" s="54"/>
-      <c r="C22" s="55"/>
-      <c r="D22" s="50"/>
-      <c r="E22" s="50"/>
+      <c r="B22" s="43"/>
+      <c r="C22" s="52"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="49"/>
       <c r="F22" s="9" t="s">
         <v>64</v>
       </c>
@@ -1860,19 +1857,19 @@
       <c r="I22" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="K22" s="43"/>
+      <c r="K22" s="45"/>
     </row>
     <row r="23" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B23" s="54" t="s">
+      <c r="B23" s="43" t="s">
         <v>65</v>
       </c>
-      <c r="C23" s="56">
+      <c r="C23" s="50">
         <v>1</v>
       </c>
-      <c r="D23" s="48" t="s">
+      <c r="D23" s="47" t="s">
         <v>90</v>
       </c>
-      <c r="E23" s="48" t="s">
+      <c r="E23" s="47" t="s">
         <v>68</v>
       </c>
       <c r="F23" s="15" t="s">
@@ -1887,13 +1884,13 @@
       <c r="I23" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="K23" s="43"/>
+      <c r="K23" s="45"/>
     </row>
     <row r="24" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B24" s="54"/>
-      <c r="C24" s="44"/>
-      <c r="D24" s="49"/>
-      <c r="E24" s="49"/>
+      <c r="B24" s="43"/>
+      <c r="C24" s="51"/>
+      <c r="D24" s="48"/>
+      <c r="E24" s="48"/>
       <c r="F24" s="2" t="s">
         <v>5</v>
       </c>
@@ -1906,13 +1903,13 @@
       <c r="I24" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="K24" s="43"/>
+      <c r="K24" s="45"/>
     </row>
     <row r="25" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B25" s="54"/>
-      <c r="C25" s="44"/>
-      <c r="D25" s="49"/>
-      <c r="E25" s="49"/>
+      <c r="B25" s="43"/>
+      <c r="C25" s="51"/>
+      <c r="D25" s="48"/>
+      <c r="E25" s="48"/>
       <c r="F25" s="2" t="s">
         <v>6</v>
       </c>
@@ -1925,13 +1922,13 @@
       <c r="I25" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="K25" s="43"/>
+      <c r="K25" s="45"/>
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B26" s="54"/>
-      <c r="C26" s="44"/>
-      <c r="D26" s="49"/>
-      <c r="E26" s="49"/>
+      <c r="B26" s="43"/>
+      <c r="C26" s="51"/>
+      <c r="D26" s="48"/>
+      <c r="E26" s="48"/>
       <c r="F26" s="2" t="s">
         <v>7</v>
       </c>
@@ -1944,13 +1941,13 @@
       <c r="I26" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="K26" s="45"/>
+      <c r="K26" s="46"/>
     </row>
     <row r="27" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B27" s="54"/>
-      <c r="C27" s="44"/>
-      <c r="D27" s="49"/>
-      <c r="E27" s="49"/>
+      <c r="B27" s="43"/>
+      <c r="C27" s="51"/>
+      <c r="D27" s="48"/>
+      <c r="E27" s="48"/>
       <c r="F27" s="2" t="s">
         <v>8</v>
       </c>
@@ -1968,14 +1965,14 @@
       </c>
     </row>
     <row r="28" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B28" s="54"/>
-      <c r="C28" s="56">
+      <c r="B28" s="43"/>
+      <c r="C28" s="50">
         <v>2</v>
       </c>
-      <c r="D28" s="48" t="s">
+      <c r="D28" s="47" t="s">
         <v>91</v>
       </c>
-      <c r="E28" s="48" t="s">
+      <c r="E28" s="47" t="s">
         <v>69</v>
       </c>
       <c r="F28" s="15" t="s">
@@ -1992,10 +1989,10 @@
       </c>
     </row>
     <row r="29" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B29" s="54"/>
-      <c r="C29" s="44"/>
-      <c r="D29" s="49"/>
-      <c r="E29" s="49"/>
+      <c r="B29" s="43"/>
+      <c r="C29" s="51"/>
+      <c r="D29" s="48"/>
+      <c r="E29" s="48"/>
       <c r="F29" s="2" t="s">
         <v>5</v>
       </c>
@@ -2010,10 +2007,10 @@
       </c>
     </row>
     <row r="30" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B30" s="54"/>
-      <c r="C30" s="44"/>
-      <c r="D30" s="49"/>
-      <c r="E30" s="49"/>
+      <c r="B30" s="43"/>
+      <c r="C30" s="51"/>
+      <c r="D30" s="48"/>
+      <c r="E30" s="48"/>
       <c r="F30" s="2" t="s">
         <v>6</v>
       </c>
@@ -2028,10 +2025,10 @@
       </c>
     </row>
     <row r="31" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B31" s="54"/>
-      <c r="C31" s="44"/>
-      <c r="D31" s="49"/>
-      <c r="E31" s="49"/>
+      <c r="B31" s="43"/>
+      <c r="C31" s="51"/>
+      <c r="D31" s="48"/>
+      <c r="E31" s="48"/>
       <c r="F31" s="2" t="s">
         <v>7</v>
       </c>
@@ -2046,10 +2043,10 @@
       </c>
     </row>
     <row r="32" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B32" s="54"/>
-      <c r="C32" s="55"/>
-      <c r="D32" s="50"/>
-      <c r="E32" s="50"/>
+      <c r="B32" s="43"/>
+      <c r="C32" s="52"/>
+      <c r="D32" s="49"/>
+      <c r="E32" s="49"/>
       <c r="F32" s="9" t="s">
         <v>8</v>
       </c>
@@ -2064,14 +2061,14 @@
       </c>
     </row>
     <row r="33" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B33" s="54"/>
-      <c r="C33" s="56">
+      <c r="B33" s="43"/>
+      <c r="C33" s="50">
         <v>3</v>
       </c>
-      <c r="D33" s="48" t="s">
+      <c r="D33" s="47" t="s">
         <v>91</v>
       </c>
-      <c r="E33" s="48" t="s">
+      <c r="E33" s="47" t="s">
         <v>69</v>
       </c>
       <c r="F33" s="15" t="s">
@@ -2086,20 +2083,20 @@
       <c r="I33" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="K33" s="57" t="s">
+      <c r="K33" s="42" t="s">
         <v>112</v>
       </c>
-      <c r="L33" s="57"/>
+      <c r="L33" s="42"/>
       <c r="M33" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="N33" s="1"/>
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B34" s="54"/>
-      <c r="C34" s="44"/>
-      <c r="D34" s="49"/>
-      <c r="E34" s="49"/>
+      <c r="B34" s="43"/>
+      <c r="C34" s="51"/>
+      <c r="D34" s="48"/>
+      <c r="E34" s="48"/>
       <c r="F34" s="2" t="s">
         <v>5</v>
       </c>
@@ -2116,17 +2113,17 @@
         <v>173</v>
       </c>
       <c r="L34" s="41" t="s">
-        <v>184</v>
+        <v>65</v>
       </c>
       <c r="M34" s="41" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="35" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B35" s="54"/>
-      <c r="C35" s="44"/>
-      <c r="D35" s="49"/>
-      <c r="E35" s="49"/>
+      <c r="B35" s="43"/>
+      <c r="C35" s="51"/>
+      <c r="D35" s="48"/>
+      <c r="E35" s="48"/>
       <c r="F35" s="2" t="s">
         <v>6</v>
       </c>
@@ -2143,17 +2140,17 @@
         <v>175</v>
       </c>
       <c r="L35" s="41" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="M35" s="41" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="36" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B36" s="54"/>
-      <c r="C36" s="44"/>
-      <c r="D36" s="49"/>
-      <c r="E36" s="49"/>
+      <c r="B36" s="43"/>
+      <c r="C36" s="51"/>
+      <c r="D36" s="48"/>
+      <c r="E36" s="48"/>
       <c r="F36" s="2" t="s">
         <v>7</v>
       </c>
@@ -2173,14 +2170,14 @@
         <v>181</v>
       </c>
       <c r="M36" s="41" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B37" s="54"/>
-      <c r="C37" s="55"/>
-      <c r="D37" s="50"/>
-      <c r="E37" s="50"/>
+      <c r="B37" s="43"/>
+      <c r="C37" s="52"/>
+      <c r="D37" s="49"/>
+      <c r="E37" s="49"/>
       <c r="F37" s="9" t="s">
         <v>8</v>
       </c>
@@ -2204,14 +2201,14 @@
       </c>
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B38" s="54"/>
-      <c r="C38" s="56">
+      <c r="B38" s="43"/>
+      <c r="C38" s="50">
         <v>6</v>
       </c>
-      <c r="D38" s="48" t="s">
+      <c r="D38" s="47" t="s">
         <v>90</v>
       </c>
-      <c r="E38" s="48" t="s">
+      <c r="E38" s="47" t="s">
         <v>68</v>
       </c>
       <c r="F38" s="15" t="s">
@@ -2233,14 +2230,14 @@
         <v>179</v>
       </c>
       <c r="M38" s="41" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="39" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B39" s="54"/>
-      <c r="C39" s="44"/>
-      <c r="D39" s="49"/>
-      <c r="E39" s="49"/>
+      <c r="B39" s="43"/>
+      <c r="C39" s="51"/>
+      <c r="D39" s="48"/>
+      <c r="E39" s="48"/>
       <c r="F39" s="2" t="s">
         <v>5</v>
       </c>
@@ -2260,14 +2257,14 @@
         <v>183</v>
       </c>
       <c r="M39" s="41" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B40" s="54"/>
-      <c r="C40" s="44"/>
-      <c r="D40" s="49"/>
-      <c r="E40" s="49"/>
+      <c r="B40" s="43"/>
+      <c r="C40" s="51"/>
+      <c r="D40" s="48"/>
+      <c r="E40" s="48"/>
       <c r="F40" s="2" t="s">
         <v>6</v>
       </c>
@@ -2284,17 +2281,17 @@
         <v>174</v>
       </c>
       <c r="L40" s="41" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M40" s="41" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B41" s="54"/>
-      <c r="C41" s="44"/>
-      <c r="D41" s="49"/>
-      <c r="E41" s="49"/>
+      <c r="B41" s="43"/>
+      <c r="C41" s="51"/>
+      <c r="D41" s="48"/>
+      <c r="E41" s="48"/>
       <c r="F41" s="2" t="s">
         <v>7</v>
       </c>
@@ -2311,17 +2308,17 @@
         <v>178</v>
       </c>
       <c r="L41" s="41" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M41" s="41" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B42" s="54"/>
-      <c r="C42" s="55"/>
-      <c r="D42" s="50"/>
-      <c r="E42" s="50"/>
+      <c r="B42" s="43"/>
+      <c r="C42" s="52"/>
+      <c r="D42" s="49"/>
+      <c r="E42" s="49"/>
       <c r="F42" s="9" t="s">
         <v>8</v>
       </c>
@@ -2341,20 +2338,20 @@
         <v>177</v>
       </c>
       <c r="M42" s="41" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="43" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B43" s="54" t="s">
+      <c r="B43" s="43" t="s">
         <v>66</v>
       </c>
-      <c r="C43" s="56">
+      <c r="C43" s="50">
         <v>1</v>
       </c>
-      <c r="D43" s="48" t="s">
+      <c r="D43" s="47" t="s">
         <v>91</v>
       </c>
-      <c r="E43" s="51" t="s">
+      <c r="E43" s="55" t="s">
         <v>92</v>
       </c>
       <c r="F43" s="15" t="s">
@@ -2371,10 +2368,10 @@
       </c>
     </row>
     <row r="44" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B44" s="54"/>
-      <c r="C44" s="44"/>
-      <c r="D44" s="49"/>
-      <c r="E44" s="52"/>
+      <c r="B44" s="43"/>
+      <c r="C44" s="51"/>
+      <c r="D44" s="48"/>
+      <c r="E44" s="56"/>
       <c r="F44" s="2" t="s">
         <v>10</v>
       </c>
@@ -2389,10 +2386,10 @@
       </c>
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B45" s="54"/>
-      <c r="C45" s="55"/>
-      <c r="D45" s="50"/>
-      <c r="E45" s="53"/>
+      <c r="B45" s="43"/>
+      <c r="C45" s="52"/>
+      <c r="D45" s="49"/>
+      <c r="E45" s="57"/>
       <c r="F45" s="9" t="s">
         <v>11</v>
       </c>
@@ -2407,14 +2404,14 @@
       </c>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B46" s="54"/>
-      <c r="C46" s="56">
+      <c r="B46" s="43"/>
+      <c r="C46" s="50">
         <v>2</v>
       </c>
-      <c r="D46" s="48" t="s">
+      <c r="D46" s="47" t="s">
         <v>91</v>
       </c>
-      <c r="E46" s="48" t="s">
+      <c r="E46" s="47" t="s">
         <v>67</v>
       </c>
       <c r="F46" s="15" t="s">
@@ -2431,10 +2428,10 @@
       </c>
     </row>
     <row r="47" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B47" s="54"/>
-      <c r="C47" s="44"/>
-      <c r="D47" s="49"/>
-      <c r="E47" s="49"/>
+      <c r="B47" s="43"/>
+      <c r="C47" s="51"/>
+      <c r="D47" s="48"/>
+      <c r="E47" s="48"/>
       <c r="F47" s="2" t="s">
         <v>10</v>
       </c>
@@ -2449,10 +2446,10 @@
       </c>
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B48" s="54"/>
-      <c r="C48" s="55"/>
-      <c r="D48" s="50"/>
-      <c r="E48" s="50"/>
+      <c r="B48" s="43"/>
+      <c r="C48" s="52"/>
+      <c r="D48" s="49"/>
+      <c r="E48" s="49"/>
       <c r="F48" s="9" t="s">
         <v>11</v>
       </c>
@@ -2467,14 +2464,14 @@
       </c>
     </row>
     <row r="49" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B49" s="54"/>
-      <c r="C49" s="44">
+      <c r="B49" s="43"/>
+      <c r="C49" s="51">
         <v>3</v>
       </c>
-      <c r="D49" s="49" t="s">
+      <c r="D49" s="48" t="s">
         <v>91</v>
       </c>
-      <c r="E49" s="49" t="s">
+      <c r="E49" s="48" t="s">
         <v>67</v>
       </c>
       <c r="F49" s="2" t="s">
@@ -2491,10 +2488,10 @@
       </c>
     </row>
     <row r="50" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B50" s="54"/>
-      <c r="C50" s="44"/>
-      <c r="D50" s="49"/>
-      <c r="E50" s="49"/>
+      <c r="B50" s="43"/>
+      <c r="C50" s="51"/>
+      <c r="D50" s="48"/>
+      <c r="E50" s="48"/>
       <c r="F50" s="2" t="s">
         <v>10</v>
       </c>
@@ -2509,10 +2506,10 @@
       </c>
     </row>
     <row r="51" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B51" s="54"/>
-      <c r="C51" s="55"/>
-      <c r="D51" s="50"/>
-      <c r="E51" s="50"/>
+      <c r="B51" s="43"/>
+      <c r="C51" s="52"/>
+      <c r="D51" s="49"/>
+      <c r="E51" s="49"/>
       <c r="F51" s="9" t="s">
         <v>11</v>
       </c>
@@ -2527,7 +2524,7 @@
       </c>
     </row>
     <row r="52" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B52" s="54" t="s">
+      <c r="B52" s="43" t="s">
         <v>83</v>
       </c>
       <c r="C52" s="18">
@@ -2555,7 +2552,7 @@
       </c>
     </row>
     <row r="53" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B53" s="54"/>
+      <c r="B53" s="43"/>
       <c r="C53" s="19">
         <v>1</v>
       </c>
@@ -2581,7 +2578,7 @@
       </c>
     </row>
     <row r="54" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B54" s="54"/>
+      <c r="B54" s="43"/>
       <c r="C54" s="19">
         <v>2</v>
       </c>
@@ -2607,7 +2604,7 @@
       </c>
     </row>
     <row r="55" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B55" s="54"/>
+      <c r="B55" s="43"/>
       <c r="C55" s="19">
         <v>3</v>
       </c>
@@ -2633,7 +2630,7 @@
       </c>
     </row>
     <row r="56" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B56" s="54"/>
+      <c r="B56" s="43"/>
       <c r="C56" s="19">
         <v>4</v>
       </c>
@@ -2659,7 +2656,7 @@
       </c>
     </row>
     <row r="57" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B57" s="54"/>
+      <c r="B57" s="43"/>
       <c r="C57" s="19">
         <v>5</v>
       </c>
@@ -2685,7 +2682,7 @@
       </c>
     </row>
     <row r="58" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B58" s="54"/>
+      <c r="B58" s="43"/>
       <c r="C58" s="19">
         <v>6</v>
       </c>
@@ -2711,7 +2708,7 @@
       </c>
     </row>
     <row r="59" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B59" s="54"/>
+      <c r="B59" s="43"/>
       <c r="C59" s="19">
         <v>7</v>
       </c>
@@ -2737,7 +2734,7 @@
       </c>
     </row>
     <row r="60" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B60" s="54"/>
+      <c r="B60" s="43"/>
       <c r="C60" s="19">
         <v>8</v>
       </c>
@@ -2763,7 +2760,7 @@
       </c>
     </row>
     <row r="61" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B61" s="54"/>
+      <c r="B61" s="43"/>
       <c r="C61" s="19">
         <v>9</v>
       </c>
@@ -2789,7 +2786,7 @@
       </c>
     </row>
     <row r="62" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B62" s="54"/>
+      <c r="B62" s="43"/>
       <c r="C62" s="19">
         <v>10</v>
       </c>
@@ -2815,7 +2812,7 @@
       </c>
     </row>
     <row r="63" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B63" s="54"/>
+      <c r="B63" s="43"/>
       <c r="C63" s="19">
         <v>11</v>
       </c>
@@ -2844,7 +2841,7 @@
       </c>
     </row>
     <row r="64" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B64" s="54"/>
+      <c r="B64" s="43"/>
       <c r="C64" s="19">
         <v>12</v>
       </c>
@@ -2873,7 +2870,7 @@
       </c>
     </row>
     <row r="65" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B65" s="54"/>
+      <c r="B65" s="43"/>
       <c r="C65" s="19">
         <v>13</v>
       </c>
@@ -2899,7 +2896,7 @@
       </c>
     </row>
     <row r="66" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B66" s="54"/>
+      <c r="B66" s="43"/>
       <c r="C66" s="19">
         <v>14</v>
       </c>
@@ -2925,7 +2922,7 @@
       </c>
     </row>
     <row r="67" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B67" s="54"/>
+      <c r="B67" s="43"/>
       <c r="C67" s="20">
         <v>15</v>
       </c>
@@ -2949,13 +2946,13 @@
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
-      <c r="J67" s="46" t="s">
+      <c r="J67" s="53" t="s">
         <v>144</v>
       </c>
-      <c r="K67" s="47"/>
+      <c r="K67" s="54"/>
     </row>
     <row r="68" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B68" s="42" t="s">
+      <c r="B68" s="44" t="s">
         <v>94</v>
       </c>
       <c r="C68" s="14" t="s">
@@ -2987,7 +2984,7 @@
       <c r="K68" s="26"/>
     </row>
     <row r="69" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B69" s="43"/>
+      <c r="B69" s="45"/>
       <c r="C69" s="6" t="s">
         <v>124</v>
       </c>
@@ -3017,7 +3014,7 @@
       <c r="K69" s="26"/>
     </row>
     <row r="70" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B70" s="43"/>
+      <c r="B70" s="45"/>
       <c r="C70" s="6" t="s">
         <v>125</v>
       </c>
@@ -3047,7 +3044,7 @@
       <c r="K70" s="26"/>
     </row>
     <row r="71" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B71" s="43"/>
+      <c r="B71" s="45"/>
       <c r="C71" s="6" t="s">
         <v>126</v>
       </c>
@@ -3077,7 +3074,7 @@
       <c r="K71" s="26"/>
     </row>
     <row r="72" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B72" s="43"/>
+      <c r="B72" s="45"/>
       <c r="C72" s="6" t="s">
         <v>127</v>
       </c>
@@ -3107,7 +3104,7 @@
       <c r="K72" s="26"/>
     </row>
     <row r="73" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B73" s="43"/>
+      <c r="B73" s="45"/>
       <c r="C73" s="6" t="s">
         <v>128</v>
       </c>
@@ -3137,7 +3134,7 @@
       <c r="K73" s="26"/>
     </row>
     <row r="74" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B74" s="43"/>
+      <c r="B74" s="45"/>
       <c r="C74" s="6" t="s">
         <v>129</v>
       </c>
@@ -3167,7 +3164,7 @@
       <c r="K74" s="26"/>
     </row>
     <row r="75" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B75" s="43"/>
+      <c r="B75" s="45"/>
       <c r="C75" s="6" t="s">
         <v>130</v>
       </c>
@@ -3197,7 +3194,7 @@
       <c r="K75" s="26"/>
     </row>
     <row r="76" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B76" s="43"/>
+      <c r="B76" s="45"/>
       <c r="C76" s="29" t="s">
         <v>170</v>
       </c>
@@ -3229,7 +3226,7 @@
       </c>
     </row>
     <row r="77" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B77" s="43"/>
+      <c r="B77" s="45"/>
       <c r="C77" s="29" t="s">
         <v>170</v>
       </c>
@@ -3261,7 +3258,7 @@
       </c>
     </row>
     <row r="78" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B78" s="43"/>
+      <c r="B78" s="45"/>
       <c r="C78" s="6" t="s">
         <v>156</v>
       </c>
@@ -3293,7 +3290,7 @@
       </c>
     </row>
     <row r="79" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B79" s="43"/>
+      <c r="B79" s="45"/>
       <c r="C79" s="6" t="s">
         <v>159</v>
       </c>
@@ -3325,7 +3322,7 @@
       </c>
     </row>
     <row r="80" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B80" s="43"/>
+      <c r="B80" s="45"/>
       <c r="C80" s="29" t="s">
         <v>164</v>
       </c>
@@ -3357,7 +3354,7 @@
       </c>
     </row>
     <row r="81" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B81" s="43"/>
+      <c r="B81" s="45"/>
       <c r="C81" s="6" t="s">
         <v>161</v>
       </c>
@@ -3390,7 +3387,7 @@
       </c>
     </row>
     <row r="82" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B82" s="43"/>
+      <c r="B82" s="45"/>
       <c r="C82" s="34"/>
       <c r="D82" s="35"/>
       <c r="E82" s="35"/>
@@ -3402,7 +3399,7 @@
       <c r="K82" s="36"/>
     </row>
     <row r="83" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B83" s="43"/>
+      <c r="B83" s="45"/>
       <c r="D83" s="15"/>
       <c r="E83" s="15"/>
       <c r="F83" s="15"/>
@@ -3412,7 +3409,7 @@
       <c r="K83" s="7"/>
     </row>
     <row r="84" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B84" s="44"/>
+      <c r="B84" s="51"/>
       <c r="C84" s="29" t="s">
         <v>160</v>
       </c>
@@ -3430,7 +3427,7 @@
       </c>
     </row>
     <row r="85" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B85" s="43"/>
+      <c r="B85" s="45"/>
       <c r="C85" s="29" t="s">
         <v>162</v>
       </c>
@@ -3451,7 +3448,7 @@
       </c>
     </row>
     <row r="86" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B86" s="45"/>
+      <c r="B86" s="46"/>
       <c r="C86" s="38" t="s">
         <v>163</v>
       </c>
@@ -3478,36 +3475,6 @@
     </row>
   </sheetData>
   <mergeCells count="46">
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="K6:K7"/>
-    <mergeCell ref="K10:K26"/>
-    <mergeCell ref="D19:D22"/>
-    <mergeCell ref="E3:E6"/>
-    <mergeCell ref="D3:D6"/>
-    <mergeCell ref="D15:D18"/>
-    <mergeCell ref="D7:D10"/>
-    <mergeCell ref="D11:D14"/>
-    <mergeCell ref="C23:C27"/>
-    <mergeCell ref="C28:C32"/>
-    <mergeCell ref="C33:C37"/>
-    <mergeCell ref="C38:C42"/>
-    <mergeCell ref="E46:E48"/>
-    <mergeCell ref="D38:D42"/>
-    <mergeCell ref="D28:D32"/>
-    <mergeCell ref="B3:B22"/>
-    <mergeCell ref="C3:C6"/>
-    <mergeCell ref="C7:C10"/>
-    <mergeCell ref="C11:C14"/>
-    <mergeCell ref="C15:C18"/>
-    <mergeCell ref="C19:C22"/>
-    <mergeCell ref="D46:D48"/>
-    <mergeCell ref="D49:D51"/>
-    <mergeCell ref="C49:C51"/>
-    <mergeCell ref="B43:B51"/>
-    <mergeCell ref="D43:D45"/>
-    <mergeCell ref="C43:C45"/>
-    <mergeCell ref="C46:C48"/>
     <mergeCell ref="B68:B86"/>
     <mergeCell ref="J67:K67"/>
     <mergeCell ref="E7:E10"/>
@@ -3524,6 +3491,36 @@
     <mergeCell ref="D23:D27"/>
     <mergeCell ref="B23:B42"/>
     <mergeCell ref="B52:B67"/>
+    <mergeCell ref="D49:D51"/>
+    <mergeCell ref="C49:C51"/>
+    <mergeCell ref="B43:B51"/>
+    <mergeCell ref="D43:D45"/>
+    <mergeCell ref="C43:C45"/>
+    <mergeCell ref="C46:C48"/>
+    <mergeCell ref="B3:B22"/>
+    <mergeCell ref="C3:C6"/>
+    <mergeCell ref="C7:C10"/>
+    <mergeCell ref="C11:C14"/>
+    <mergeCell ref="C15:C18"/>
+    <mergeCell ref="C19:C22"/>
+    <mergeCell ref="C23:C27"/>
+    <mergeCell ref="C28:C32"/>
+    <mergeCell ref="C33:C37"/>
+    <mergeCell ref="C38:C42"/>
+    <mergeCell ref="E46:E48"/>
+    <mergeCell ref="D38:D42"/>
+    <mergeCell ref="D28:D32"/>
+    <mergeCell ref="D46:D48"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="K6:K7"/>
+    <mergeCell ref="K10:K26"/>
+    <mergeCell ref="D19:D22"/>
+    <mergeCell ref="E3:E6"/>
+    <mergeCell ref="D3:D6"/>
+    <mergeCell ref="D15:D18"/>
+    <mergeCell ref="D7:D10"/>
+    <mergeCell ref="D11:D14"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: add acceleromter high g, fix communication protocole mapping excel, fix beacon i2c connector (id i2c channel) and add footprint/symbole accelerometer
</commit_message>
<xml_diff>
--- a/ODB_V3/Hardware/Kicad/STM32F412ZGT6_Interfaces.xlsx
+++ b/ODB_V3/Hardware/Kicad/STM32F412ZGT6_Interfaces.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gagno\OneDrive\Documents\ULaval\GAUL\ODB2\Ordinateur-de-bord\ODB_V3\Hardware\Kicad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0191D53-32D2-4AB7-B999-89BFA3C6C21B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2877C714-07AB-438B-88FD-65706A253676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2490" yWindow="3015" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="193">
   <si>
     <t>Interface</t>
   </si>
@@ -590,9 +590,6 @@
     <t>I2C2</t>
   </si>
   <si>
-    <t>SPI4</t>
-  </si>
-  <si>
     <t>SPI5</t>
   </si>
   <si>
@@ -609,6 +606,12 @@
   </si>
   <si>
     <t>6,25Mbit/s</t>
+  </si>
+  <si>
+    <t>I2C1</t>
+  </si>
+  <si>
+    <t>QuadSPI</t>
   </si>
 </sst>
 </file>
@@ -964,21 +967,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -986,21 +992,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1011,6 +1002,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1415,16 +1418,16 @@
       </c>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="54" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="50">
+      <c r="C3" s="56">
         <v>1</v>
       </c>
-      <c r="D3" s="47" t="s">
+      <c r="D3" s="48" t="s">
         <v>90</v>
       </c>
-      <c r="E3" s="47" t="s">
+      <c r="E3" s="48" t="s">
         <v>70</v>
       </c>
       <c r="F3" s="15" t="s">
@@ -1439,7 +1442,7 @@
       <c r="I3" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="K3" s="43" t="s">
+      <c r="K3" s="54" t="s">
         <v>94</v>
       </c>
       <c r="L3" s="22" t="s">
@@ -1447,10 +1450,10 @@
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B4" s="43"/>
-      <c r="C4" s="51"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="48"/>
+      <c r="B4" s="54"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="49"/>
+      <c r="E4" s="49"/>
       <c r="F4" s="2" t="s">
         <v>2</v>
       </c>
@@ -1463,16 +1466,16 @@
       <c r="I4" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="K4" s="43"/>
+      <c r="K4" s="54"/>
       <c r="L4" s="23" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="43"/>
-      <c r="C5" s="51"/>
-      <c r="D5" s="48"/>
-      <c r="E5" s="48"/>
+      <c r="B5" s="54"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="49"/>
       <c r="F5" s="2" t="s">
         <v>3</v>
       </c>
@@ -1493,10 +1496,10 @@
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B6" s="43"/>
-      <c r="C6" s="51"/>
-      <c r="D6" s="48"/>
-      <c r="E6" s="48"/>
+      <c r="B6" s="54"/>
+      <c r="C6" s="44"/>
+      <c r="D6" s="49"/>
+      <c r="E6" s="49"/>
       <c r="F6" s="2" t="s">
         <v>64</v>
       </c>
@@ -1509,7 +1512,7 @@
       <c r="I6" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="K6" s="43" t="s">
+      <c r="K6" s="54" t="s">
         <v>101</v>
       </c>
       <c r="L6" s="22" t="s">
@@ -1517,14 +1520,14 @@
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B7" s="43"/>
-      <c r="C7" s="50">
+      <c r="B7" s="54"/>
+      <c r="C7" s="56">
         <v>2</v>
       </c>
-      <c r="D7" s="47" t="s">
+      <c r="D7" s="48" t="s">
         <v>91</v>
       </c>
-      <c r="E7" s="47" t="s">
+      <c r="E7" s="48" t="s">
         <v>71</v>
       </c>
       <c r="F7" s="15" t="s">
@@ -1539,16 +1542,16 @@
       <c r="I7" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="K7" s="43"/>
+      <c r="K7" s="54"/>
       <c r="L7" s="23" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B8" s="43"/>
-      <c r="C8" s="51"/>
-      <c r="D8" s="48"/>
-      <c r="E8" s="48"/>
+      <c r="B8" s="54"/>
+      <c r="C8" s="44"/>
+      <c r="D8" s="49"/>
+      <c r="E8" s="49"/>
       <c r="F8" s="2" t="s">
         <v>2</v>
       </c>
@@ -1569,10 +1572,10 @@
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B9" s="43"/>
-      <c r="C9" s="51"/>
-      <c r="D9" s="48"/>
-      <c r="E9" s="48"/>
+      <c r="B9" s="54"/>
+      <c r="C9" s="44"/>
+      <c r="D9" s="49"/>
+      <c r="E9" s="49"/>
       <c r="F9" s="2" t="s">
         <v>3</v>
       </c>
@@ -1593,10 +1596,10 @@
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B10" s="43"/>
-      <c r="C10" s="52"/>
-      <c r="D10" s="49"/>
-      <c r="E10" s="49"/>
+      <c r="B10" s="54"/>
+      <c r="C10" s="55"/>
+      <c r="D10" s="50"/>
+      <c r="E10" s="50"/>
       <c r="F10" s="9" t="s">
         <v>64</v>
       </c>
@@ -1609,19 +1612,19 @@
       <c r="I10" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="K10" s="44" t="s">
+      <c r="K10" s="42" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="43"/>
-      <c r="C11" s="50">
+      <c r="B11" s="54"/>
+      <c r="C11" s="56">
         <v>3</v>
       </c>
-      <c r="D11" s="47" t="s">
+      <c r="D11" s="48" t="s">
         <v>91</v>
       </c>
-      <c r="E11" s="47" t="s">
+      <c r="E11" s="48" t="s">
         <v>71</v>
       </c>
       <c r="F11" s="15" t="s">
@@ -1636,13 +1639,13 @@
       <c r="I11" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="K11" s="45"/>
+      <c r="K11" s="43"/>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B12" s="43"/>
-      <c r="C12" s="51"/>
-      <c r="D12" s="48"/>
-      <c r="E12" s="48"/>
+      <c r="B12" s="54"/>
+      <c r="C12" s="44"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="49"/>
       <c r="F12" s="2" t="s">
         <v>2</v>
       </c>
@@ -1655,13 +1658,13 @@
       <c r="I12" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="K12" s="45"/>
+      <c r="K12" s="43"/>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B13" s="43"/>
-      <c r="C13" s="51"/>
-      <c r="D13" s="48"/>
-      <c r="E13" s="48"/>
+      <c r="B13" s="54"/>
+      <c r="C13" s="44"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="49"/>
       <c r="F13" s="2" t="s">
         <v>3</v>
       </c>
@@ -1674,13 +1677,13 @@
       <c r="I13" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="K13" s="45"/>
+      <c r="K13" s="43"/>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B14" s="43"/>
-      <c r="C14" s="52"/>
-      <c r="D14" s="49"/>
-      <c r="E14" s="49"/>
+      <c r="B14" s="54"/>
+      <c r="C14" s="55"/>
+      <c r="D14" s="50"/>
+      <c r="E14" s="50"/>
       <c r="F14" s="9" t="s">
         <v>64</v>
       </c>
@@ -1693,17 +1696,17 @@
       <c r="I14" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="K14" s="45"/>
+      <c r="K14" s="43"/>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B15" s="43"/>
-      <c r="C15" s="50">
+      <c r="B15" s="54"/>
+      <c r="C15" s="56">
         <v>4</v>
       </c>
-      <c r="D15" s="47" t="s">
+      <c r="D15" s="48" t="s">
         <v>90</v>
       </c>
-      <c r="E15" s="47" t="s">
+      <c r="E15" s="48" t="s">
         <v>70</v>
       </c>
       <c r="F15" s="15" t="s">
@@ -1718,13 +1721,13 @@
       <c r="I15" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="K15" s="45"/>
+      <c r="K15" s="43"/>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B16" s="43"/>
-      <c r="C16" s="51"/>
-      <c r="D16" s="48"/>
-      <c r="E16" s="48"/>
+      <c r="B16" s="54"/>
+      <c r="C16" s="44"/>
+      <c r="D16" s="49"/>
+      <c r="E16" s="49"/>
       <c r="F16" s="2" t="s">
         <v>2</v>
       </c>
@@ -1737,13 +1740,13 @@
       <c r="I16" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="K16" s="45"/>
+      <c r="K16" s="43"/>
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B17" s="43"/>
-      <c r="C17" s="51"/>
-      <c r="D17" s="48"/>
-      <c r="E17" s="48"/>
+      <c r="B17" s="54"/>
+      <c r="C17" s="44"/>
+      <c r="D17" s="49"/>
+      <c r="E17" s="49"/>
       <c r="F17" s="2" t="s">
         <v>3</v>
       </c>
@@ -1756,13 +1759,13 @@
       <c r="I17" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="K17" s="45"/>
+      <c r="K17" s="43"/>
     </row>
     <row r="18" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B18" s="43"/>
-      <c r="C18" s="52"/>
-      <c r="D18" s="49"/>
-      <c r="E18" s="49"/>
+      <c r="B18" s="54"/>
+      <c r="C18" s="55"/>
+      <c r="D18" s="50"/>
+      <c r="E18" s="50"/>
       <c r="F18" s="9" t="s">
         <v>64</v>
       </c>
@@ -1775,17 +1778,17 @@
       <c r="I18" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="K18" s="45"/>
+      <c r="K18" s="43"/>
     </row>
     <row r="19" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B19" s="43"/>
-      <c r="C19" s="50">
+      <c r="B19" s="54"/>
+      <c r="C19" s="56">
         <v>5</v>
       </c>
-      <c r="D19" s="47" t="s">
+      <c r="D19" s="48" t="s">
         <v>90</v>
       </c>
-      <c r="E19" s="47" t="s">
+      <c r="E19" s="48" t="s">
         <v>70</v>
       </c>
       <c r="F19" s="15" t="s">
@@ -1800,13 +1803,13 @@
       <c r="I19" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="K19" s="45"/>
+      <c r="K19" s="43"/>
     </row>
     <row r="20" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B20" s="43"/>
-      <c r="C20" s="51"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="48"/>
+      <c r="B20" s="54"/>
+      <c r="C20" s="44"/>
+      <c r="D20" s="49"/>
+      <c r="E20" s="49"/>
       <c r="F20" s="2" t="s">
         <v>2</v>
       </c>
@@ -1819,13 +1822,13 @@
       <c r="I20" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="K20" s="45"/>
+      <c r="K20" s="43"/>
     </row>
     <row r="21" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B21" s="43"/>
-      <c r="C21" s="51"/>
-      <c r="D21" s="48"/>
-      <c r="E21" s="48"/>
+      <c r="B21" s="54"/>
+      <c r="C21" s="44"/>
+      <c r="D21" s="49"/>
+      <c r="E21" s="49"/>
       <c r="F21" s="2" t="s">
         <v>3</v>
       </c>
@@ -1838,13 +1841,13 @@
       <c r="I21" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="K21" s="45"/>
+      <c r="K21" s="43"/>
     </row>
     <row r="22" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B22" s="43"/>
-      <c r="C22" s="52"/>
-      <c r="D22" s="49"/>
-      <c r="E22" s="49"/>
+      <c r="B22" s="54"/>
+      <c r="C22" s="55"/>
+      <c r="D22" s="50"/>
+      <c r="E22" s="50"/>
       <c r="F22" s="9" t="s">
         <v>64</v>
       </c>
@@ -1857,19 +1860,19 @@
       <c r="I22" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="K22" s="45"/>
+      <c r="K22" s="43"/>
     </row>
     <row r="23" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B23" s="43" t="s">
+      <c r="B23" s="54" t="s">
         <v>65</v>
       </c>
-      <c r="C23" s="50">
+      <c r="C23" s="56">
         <v>1</v>
       </c>
-      <c r="D23" s="47" t="s">
+      <c r="D23" s="48" t="s">
         <v>90</v>
       </c>
-      <c r="E23" s="47" t="s">
+      <c r="E23" s="48" t="s">
         <v>68</v>
       </c>
       <c r="F23" s="15" t="s">
@@ -1884,13 +1887,13 @@
       <c r="I23" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="K23" s="45"/>
+      <c r="K23" s="43"/>
     </row>
     <row r="24" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B24" s="43"/>
-      <c r="C24" s="51"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="48"/>
+      <c r="B24" s="54"/>
+      <c r="C24" s="44"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="49"/>
       <c r="F24" s="2" t="s">
         <v>5</v>
       </c>
@@ -1903,13 +1906,13 @@
       <c r="I24" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="K24" s="45"/>
+      <c r="K24" s="43"/>
     </row>
     <row r="25" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B25" s="43"/>
-      <c r="C25" s="51"/>
-      <c r="D25" s="48"/>
-      <c r="E25" s="48"/>
+      <c r="B25" s="54"/>
+      <c r="C25" s="44"/>
+      <c r="D25" s="49"/>
+      <c r="E25" s="49"/>
       <c r="F25" s="2" t="s">
         <v>6</v>
       </c>
@@ -1922,13 +1925,13 @@
       <c r="I25" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="K25" s="45"/>
+      <c r="K25" s="43"/>
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B26" s="43"/>
-      <c r="C26" s="51"/>
-      <c r="D26" s="48"/>
-      <c r="E26" s="48"/>
+      <c r="B26" s="54"/>
+      <c r="C26" s="44"/>
+      <c r="D26" s="49"/>
+      <c r="E26" s="49"/>
       <c r="F26" s="2" t="s">
         <v>7</v>
       </c>
@@ -1941,13 +1944,13 @@
       <c r="I26" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="K26" s="46"/>
+      <c r="K26" s="45"/>
     </row>
     <row r="27" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B27" s="43"/>
-      <c r="C27" s="51"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="48"/>
+      <c r="B27" s="54"/>
+      <c r="C27" s="44"/>
+      <c r="D27" s="49"/>
+      <c r="E27" s="49"/>
       <c r="F27" s="2" t="s">
         <v>8</v>
       </c>
@@ -1965,14 +1968,14 @@
       </c>
     </row>
     <row r="28" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B28" s="43"/>
-      <c r="C28" s="50">
+      <c r="B28" s="54"/>
+      <c r="C28" s="56">
         <v>2</v>
       </c>
-      <c r="D28" s="47" t="s">
+      <c r="D28" s="48" t="s">
         <v>91</v>
       </c>
-      <c r="E28" s="47" t="s">
+      <c r="E28" s="48" t="s">
         <v>69</v>
       </c>
       <c r="F28" s="15" t="s">
@@ -1989,10 +1992,10 @@
       </c>
     </row>
     <row r="29" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B29" s="43"/>
-      <c r="C29" s="51"/>
-      <c r="D29" s="48"/>
-      <c r="E29" s="48"/>
+      <c r="B29" s="54"/>
+      <c r="C29" s="44"/>
+      <c r="D29" s="49"/>
+      <c r="E29" s="49"/>
       <c r="F29" s="2" t="s">
         <v>5</v>
       </c>
@@ -2007,10 +2010,10 @@
       </c>
     </row>
     <row r="30" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B30" s="43"/>
-      <c r="C30" s="51"/>
-      <c r="D30" s="48"/>
-      <c r="E30" s="48"/>
+      <c r="B30" s="54"/>
+      <c r="C30" s="44"/>
+      <c r="D30" s="49"/>
+      <c r="E30" s="49"/>
       <c r="F30" s="2" t="s">
         <v>6</v>
       </c>
@@ -2025,10 +2028,10 @@
       </c>
     </row>
     <row r="31" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B31" s="43"/>
-      <c r="C31" s="51"/>
-      <c r="D31" s="48"/>
-      <c r="E31" s="48"/>
+      <c r="B31" s="54"/>
+      <c r="C31" s="44"/>
+      <c r="D31" s="49"/>
+      <c r="E31" s="49"/>
       <c r="F31" s="2" t="s">
         <v>7</v>
       </c>
@@ -2043,10 +2046,10 @@
       </c>
     </row>
     <row r="32" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B32" s="43"/>
-      <c r="C32" s="52"/>
-      <c r="D32" s="49"/>
-      <c r="E32" s="49"/>
+      <c r="B32" s="54"/>
+      <c r="C32" s="55"/>
+      <c r="D32" s="50"/>
+      <c r="E32" s="50"/>
       <c r="F32" s="9" t="s">
         <v>8</v>
       </c>
@@ -2061,14 +2064,14 @@
       </c>
     </row>
     <row r="33" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B33" s="43"/>
-      <c r="C33" s="50">
+      <c r="B33" s="54"/>
+      <c r="C33" s="56">
         <v>3</v>
       </c>
-      <c r="D33" s="47" t="s">
+      <c r="D33" s="48" t="s">
         <v>91</v>
       </c>
-      <c r="E33" s="47" t="s">
+      <c r="E33" s="48" t="s">
         <v>69</v>
       </c>
       <c r="F33" s="15" t="s">
@@ -2083,20 +2086,20 @@
       <c r="I33" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="K33" s="42" t="s">
+      <c r="K33" s="57" t="s">
         <v>112</v>
       </c>
-      <c r="L33" s="42"/>
+      <c r="L33" s="57"/>
       <c r="M33" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="N33" s="1"/>
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B34" s="43"/>
-      <c r="C34" s="51"/>
-      <c r="D34" s="48"/>
-      <c r="E34" s="48"/>
+      <c r="B34" s="54"/>
+      <c r="C34" s="44"/>
+      <c r="D34" s="49"/>
+      <c r="E34" s="49"/>
       <c r="F34" s="2" t="s">
         <v>5</v>
       </c>
@@ -2113,17 +2116,17 @@
         <v>173</v>
       </c>
       <c r="L34" s="41" t="s">
-        <v>65</v>
+        <v>181</v>
       </c>
       <c r="M34" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="35" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B35" s="43"/>
-      <c r="C35" s="51"/>
-      <c r="D35" s="48"/>
-      <c r="E35" s="48"/>
+      <c r="B35" s="54"/>
+      <c r="C35" s="44"/>
+      <c r="D35" s="49"/>
+      <c r="E35" s="49"/>
       <c r="F35" s="2" t="s">
         <v>6</v>
       </c>
@@ -2140,17 +2143,17 @@
         <v>175</v>
       </c>
       <c r="L35" s="41" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="M35" s="41" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="36" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B36" s="43"/>
-      <c r="C36" s="51"/>
-      <c r="D36" s="48"/>
-      <c r="E36" s="48"/>
+      <c r="B36" s="54"/>
+      <c r="C36" s="44"/>
+      <c r="D36" s="49"/>
+      <c r="E36" s="49"/>
       <c r="F36" s="2" t="s">
         <v>7</v>
       </c>
@@ -2167,17 +2170,17 @@
         <v>180</v>
       </c>
       <c r="L36" s="41" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="M36" s="41" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B37" s="43"/>
-      <c r="C37" s="52"/>
-      <c r="D37" s="49"/>
-      <c r="E37" s="49"/>
+      <c r="B37" s="54"/>
+      <c r="C37" s="55"/>
+      <c r="D37" s="50"/>
+      <c r="E37" s="50"/>
       <c r="F37" s="9" t="s">
         <v>8</v>
       </c>
@@ -2201,14 +2204,14 @@
       </c>
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B38" s="43"/>
-      <c r="C38" s="50">
+      <c r="B38" s="54"/>
+      <c r="C38" s="56">
         <v>6</v>
       </c>
-      <c r="D38" s="47" t="s">
+      <c r="D38" s="48" t="s">
         <v>90</v>
       </c>
-      <c r="E38" s="47" t="s">
+      <c r="E38" s="48" t="s">
         <v>68</v>
       </c>
       <c r="F38" s="15" t="s">
@@ -2230,14 +2233,14 @@
         <v>179</v>
       </c>
       <c r="M38" s="41" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="39" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B39" s="43"/>
-      <c r="C39" s="51"/>
-      <c r="D39" s="48"/>
-      <c r="E39" s="48"/>
+      <c r="B39" s="54"/>
+      <c r="C39" s="44"/>
+      <c r="D39" s="49"/>
+      <c r="E39" s="49"/>
       <c r="F39" s="2" t="s">
         <v>5</v>
       </c>
@@ -2254,17 +2257,17 @@
         <v>115</v>
       </c>
       <c r="L39" s="41" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="M39" s="41" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B40" s="43"/>
-      <c r="C40" s="51"/>
-      <c r="D40" s="48"/>
-      <c r="E40" s="48"/>
+      <c r="B40" s="54"/>
+      <c r="C40" s="44"/>
+      <c r="D40" s="49"/>
+      <c r="E40" s="49"/>
       <c r="F40" s="2" t="s">
         <v>6</v>
       </c>
@@ -2281,17 +2284,17 @@
         <v>174</v>
       </c>
       <c r="L40" s="41" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="M40" s="41" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B41" s="43"/>
-      <c r="C41" s="51"/>
-      <c r="D41" s="48"/>
-      <c r="E41" s="48"/>
+      <c r="B41" s="54"/>
+      <c r="C41" s="44"/>
+      <c r="D41" s="49"/>
+      <c r="E41" s="49"/>
       <c r="F41" s="2" t="s">
         <v>7</v>
       </c>
@@ -2308,17 +2311,17 @@
         <v>178</v>
       </c>
       <c r="L41" s="41" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M41" s="41" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B42" s="43"/>
-      <c r="C42" s="52"/>
-      <c r="D42" s="49"/>
-      <c r="E42" s="49"/>
+      <c r="B42" s="54"/>
+      <c r="C42" s="55"/>
+      <c r="D42" s="50"/>
+      <c r="E42" s="50"/>
       <c r="F42" s="9" t="s">
         <v>8</v>
       </c>
@@ -2335,23 +2338,23 @@
         <v>176</v>
       </c>
       <c r="L42" s="41" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="M42" s="41" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="43" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B43" s="43" t="s">
+      <c r="B43" s="54" t="s">
         <v>66</v>
       </c>
-      <c r="C43" s="50">
+      <c r="C43" s="56">
         <v>1</v>
       </c>
-      <c r="D43" s="47" t="s">
+      <c r="D43" s="48" t="s">
         <v>91</v>
       </c>
-      <c r="E43" s="55" t="s">
+      <c r="E43" s="51" t="s">
         <v>92</v>
       </c>
       <c r="F43" s="15" t="s">
@@ -2368,10 +2371,10 @@
       </c>
     </row>
     <row r="44" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B44" s="43"/>
-      <c r="C44" s="51"/>
-      <c r="D44" s="48"/>
-      <c r="E44" s="56"/>
+      <c r="B44" s="54"/>
+      <c r="C44" s="44"/>
+      <c r="D44" s="49"/>
+      <c r="E44" s="52"/>
       <c r="F44" s="2" t="s">
         <v>10</v>
       </c>
@@ -2386,10 +2389,10 @@
       </c>
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B45" s="43"/>
-      <c r="C45" s="52"/>
-      <c r="D45" s="49"/>
-      <c r="E45" s="57"/>
+      <c r="B45" s="54"/>
+      <c r="C45" s="55"/>
+      <c r="D45" s="50"/>
+      <c r="E45" s="53"/>
       <c r="F45" s="9" t="s">
         <v>11</v>
       </c>
@@ -2404,14 +2407,14 @@
       </c>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B46" s="43"/>
-      <c r="C46" s="50">
+      <c r="B46" s="54"/>
+      <c r="C46" s="56">
         <v>2</v>
       </c>
-      <c r="D46" s="47" t="s">
+      <c r="D46" s="48" t="s">
         <v>91</v>
       </c>
-      <c r="E46" s="47" t="s">
+      <c r="E46" s="48" t="s">
         <v>67</v>
       </c>
       <c r="F46" s="15" t="s">
@@ -2428,10 +2431,10 @@
       </c>
     </row>
     <row r="47" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B47" s="43"/>
-      <c r="C47" s="51"/>
-      <c r="D47" s="48"/>
-      <c r="E47" s="48"/>
+      <c r="B47" s="54"/>
+      <c r="C47" s="44"/>
+      <c r="D47" s="49"/>
+      <c r="E47" s="49"/>
       <c r="F47" s="2" t="s">
         <v>10</v>
       </c>
@@ -2446,10 +2449,10 @@
       </c>
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B48" s="43"/>
-      <c r="C48" s="52"/>
-      <c r="D48" s="49"/>
-      <c r="E48" s="49"/>
+      <c r="B48" s="54"/>
+      <c r="C48" s="55"/>
+      <c r="D48" s="50"/>
+      <c r="E48" s="50"/>
       <c r="F48" s="9" t="s">
         <v>11</v>
       </c>
@@ -2464,14 +2467,14 @@
       </c>
     </row>
     <row r="49" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B49" s="43"/>
-      <c r="C49" s="51">
+      <c r="B49" s="54"/>
+      <c r="C49" s="44">
         <v>3</v>
       </c>
-      <c r="D49" s="48" t="s">
+      <c r="D49" s="49" t="s">
         <v>91</v>
       </c>
-      <c r="E49" s="48" t="s">
+      <c r="E49" s="49" t="s">
         <v>67</v>
       </c>
       <c r="F49" s="2" t="s">
@@ -2488,10 +2491,10 @@
       </c>
     </row>
     <row r="50" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B50" s="43"/>
-      <c r="C50" s="51"/>
-      <c r="D50" s="48"/>
-      <c r="E50" s="48"/>
+      <c r="B50" s="54"/>
+      <c r="C50" s="44"/>
+      <c r="D50" s="49"/>
+      <c r="E50" s="49"/>
       <c r="F50" s="2" t="s">
         <v>10</v>
       </c>
@@ -2506,10 +2509,10 @@
       </c>
     </row>
     <row r="51" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B51" s="43"/>
-      <c r="C51" s="52"/>
-      <c r="D51" s="49"/>
-      <c r="E51" s="49"/>
+      <c r="B51" s="54"/>
+      <c r="C51" s="55"/>
+      <c r="D51" s="50"/>
+      <c r="E51" s="50"/>
       <c r="F51" s="9" t="s">
         <v>11</v>
       </c>
@@ -2524,7 +2527,7 @@
       </c>
     </row>
     <row r="52" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B52" s="43" t="s">
+      <c r="B52" s="54" t="s">
         <v>83</v>
       </c>
       <c r="C52" s="18">
@@ -2552,7 +2555,7 @@
       </c>
     </row>
     <row r="53" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B53" s="43"/>
+      <c r="B53" s="54"/>
       <c r="C53" s="19">
         <v>1</v>
       </c>
@@ -2578,7 +2581,7 @@
       </c>
     </row>
     <row r="54" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B54" s="43"/>
+      <c r="B54" s="54"/>
       <c r="C54" s="19">
         <v>2</v>
       </c>
@@ -2604,7 +2607,7 @@
       </c>
     </row>
     <row r="55" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B55" s="43"/>
+      <c r="B55" s="54"/>
       <c r="C55" s="19">
         <v>3</v>
       </c>
@@ -2630,7 +2633,7 @@
       </c>
     </row>
     <row r="56" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B56" s="43"/>
+      <c r="B56" s="54"/>
       <c r="C56" s="19">
         <v>4</v>
       </c>
@@ -2656,7 +2659,7 @@
       </c>
     </row>
     <row r="57" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B57" s="43"/>
+      <c r="B57" s="54"/>
       <c r="C57" s="19">
         <v>5</v>
       </c>
@@ -2682,7 +2685,7 @@
       </c>
     </row>
     <row r="58" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B58" s="43"/>
+      <c r="B58" s="54"/>
       <c r="C58" s="19">
         <v>6</v>
       </c>
@@ -2708,7 +2711,7 @@
       </c>
     </row>
     <row r="59" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B59" s="43"/>
+      <c r="B59" s="54"/>
       <c r="C59" s="19">
         <v>7</v>
       </c>
@@ -2734,7 +2737,7 @@
       </c>
     </row>
     <row r="60" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B60" s="43"/>
+      <c r="B60" s="54"/>
       <c r="C60" s="19">
         <v>8</v>
       </c>
@@ -2760,7 +2763,7 @@
       </c>
     </row>
     <row r="61" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B61" s="43"/>
+      <c r="B61" s="54"/>
       <c r="C61" s="19">
         <v>9</v>
       </c>
@@ -2786,7 +2789,7 @@
       </c>
     </row>
     <row r="62" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B62" s="43"/>
+      <c r="B62" s="54"/>
       <c r="C62" s="19">
         <v>10</v>
       </c>
@@ -2812,7 +2815,7 @@
       </c>
     </row>
     <row r="63" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B63" s="43"/>
+      <c r="B63" s="54"/>
       <c r="C63" s="19">
         <v>11</v>
       </c>
@@ -2841,7 +2844,7 @@
       </c>
     </row>
     <row r="64" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B64" s="43"/>
+      <c r="B64" s="54"/>
       <c r="C64" s="19">
         <v>12</v>
       </c>
@@ -2870,7 +2873,7 @@
       </c>
     </row>
     <row r="65" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B65" s="43"/>
+      <c r="B65" s="54"/>
       <c r="C65" s="19">
         <v>13</v>
       </c>
@@ -2896,7 +2899,7 @@
       </c>
     </row>
     <row r="66" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B66" s="43"/>
+      <c r="B66" s="54"/>
       <c r="C66" s="19">
         <v>14</v>
       </c>
@@ -2922,7 +2925,7 @@
       </c>
     </row>
     <row r="67" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B67" s="43"/>
+      <c r="B67" s="54"/>
       <c r="C67" s="20">
         <v>15</v>
       </c>
@@ -2946,13 +2949,13 @@
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
-      <c r="J67" s="53" t="s">
+      <c r="J67" s="46" t="s">
         <v>144</v>
       </c>
-      <c r="K67" s="54"/>
+      <c r="K67" s="47"/>
     </row>
     <row r="68" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B68" s="44" t="s">
+      <c r="B68" s="42" t="s">
         <v>94</v>
       </c>
       <c r="C68" s="14" t="s">
@@ -2984,7 +2987,7 @@
       <c r="K68" s="26"/>
     </row>
     <row r="69" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B69" s="45"/>
+      <c r="B69" s="43"/>
       <c r="C69" s="6" t="s">
         <v>124</v>
       </c>
@@ -3014,7 +3017,7 @@
       <c r="K69" s="26"/>
     </row>
     <row r="70" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B70" s="45"/>
+      <c r="B70" s="43"/>
       <c r="C70" s="6" t="s">
         <v>125</v>
       </c>
@@ -3044,7 +3047,7 @@
       <c r="K70" s="26"/>
     </row>
     <row r="71" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B71" s="45"/>
+      <c r="B71" s="43"/>
       <c r="C71" s="6" t="s">
         <v>126</v>
       </c>
@@ -3074,7 +3077,7 @@
       <c r="K71" s="26"/>
     </row>
     <row r="72" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B72" s="45"/>
+      <c r="B72" s="43"/>
       <c r="C72" s="6" t="s">
         <v>127</v>
       </c>
@@ -3104,7 +3107,7 @@
       <c r="K72" s="26"/>
     </row>
     <row r="73" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B73" s="45"/>
+      <c r="B73" s="43"/>
       <c r="C73" s="6" t="s">
         <v>128</v>
       </c>
@@ -3134,7 +3137,7 @@
       <c r="K73" s="26"/>
     </row>
     <row r="74" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B74" s="45"/>
+      <c r="B74" s="43"/>
       <c r="C74" s="6" t="s">
         <v>129</v>
       </c>
@@ -3164,7 +3167,7 @@
       <c r="K74" s="26"/>
     </row>
     <row r="75" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B75" s="45"/>
+      <c r="B75" s="43"/>
       <c r="C75" s="6" t="s">
         <v>130</v>
       </c>
@@ -3194,7 +3197,7 @@
       <c r="K75" s="26"/>
     </row>
     <row r="76" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B76" s="45"/>
+      <c r="B76" s="43"/>
       <c r="C76" s="29" t="s">
         <v>170</v>
       </c>
@@ -3226,7 +3229,7 @@
       </c>
     </row>
     <row r="77" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B77" s="45"/>
+      <c r="B77" s="43"/>
       <c r="C77" s="29" t="s">
         <v>170</v>
       </c>
@@ -3258,7 +3261,7 @@
       </c>
     </row>
     <row r="78" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B78" s="45"/>
+      <c r="B78" s="43"/>
       <c r="C78" s="6" t="s">
         <v>156</v>
       </c>
@@ -3290,7 +3293,7 @@
       </c>
     </row>
     <row r="79" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B79" s="45"/>
+      <c r="B79" s="43"/>
       <c r="C79" s="6" t="s">
         <v>159</v>
       </c>
@@ -3322,7 +3325,7 @@
       </c>
     </row>
     <row r="80" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B80" s="45"/>
+      <c r="B80" s="43"/>
       <c r="C80" s="29" t="s">
         <v>164</v>
       </c>
@@ -3354,7 +3357,7 @@
       </c>
     </row>
     <row r="81" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B81" s="45"/>
+      <c r="B81" s="43"/>
       <c r="C81" s="6" t="s">
         <v>161</v>
       </c>
@@ -3387,7 +3390,7 @@
       </c>
     </row>
     <row r="82" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B82" s="45"/>
+      <c r="B82" s="43"/>
       <c r="C82" s="34"/>
       <c r="D82" s="35"/>
       <c r="E82" s="35"/>
@@ -3399,7 +3402,7 @@
       <c r="K82" s="36"/>
     </row>
     <row r="83" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B83" s="45"/>
+      <c r="B83" s="43"/>
       <c r="D83" s="15"/>
       <c r="E83" s="15"/>
       <c r="F83" s="15"/>
@@ -3409,7 +3412,7 @@
       <c r="K83" s="7"/>
     </row>
     <row r="84" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B84" s="51"/>
+      <c r="B84" s="44"/>
       <c r="C84" s="29" t="s">
         <v>160</v>
       </c>
@@ -3427,7 +3430,7 @@
       </c>
     </row>
     <row r="85" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B85" s="45"/>
+      <c r="B85" s="43"/>
       <c r="C85" s="29" t="s">
         <v>162</v>
       </c>
@@ -3448,7 +3451,7 @@
       </c>
     </row>
     <row r="86" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B86" s="46"/>
+      <c r="B86" s="45"/>
       <c r="C86" s="38" t="s">
         <v>163</v>
       </c>
@@ -3475,6 +3478,36 @@
     </row>
   </sheetData>
   <mergeCells count="46">
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="K6:K7"/>
+    <mergeCell ref="K10:K26"/>
+    <mergeCell ref="D19:D22"/>
+    <mergeCell ref="E3:E6"/>
+    <mergeCell ref="D3:D6"/>
+    <mergeCell ref="D15:D18"/>
+    <mergeCell ref="D7:D10"/>
+    <mergeCell ref="D11:D14"/>
+    <mergeCell ref="C23:C27"/>
+    <mergeCell ref="C28:C32"/>
+    <mergeCell ref="C33:C37"/>
+    <mergeCell ref="C38:C42"/>
+    <mergeCell ref="E46:E48"/>
+    <mergeCell ref="D38:D42"/>
+    <mergeCell ref="D28:D32"/>
+    <mergeCell ref="D46:D48"/>
+    <mergeCell ref="B3:B22"/>
+    <mergeCell ref="C3:C6"/>
+    <mergeCell ref="C7:C10"/>
+    <mergeCell ref="C11:C14"/>
+    <mergeCell ref="C15:C18"/>
+    <mergeCell ref="C19:C22"/>
+    <mergeCell ref="D49:D51"/>
+    <mergeCell ref="C49:C51"/>
+    <mergeCell ref="B43:B51"/>
+    <mergeCell ref="D43:D45"/>
+    <mergeCell ref="C43:C45"/>
+    <mergeCell ref="C46:C48"/>
     <mergeCell ref="B68:B86"/>
     <mergeCell ref="J67:K67"/>
     <mergeCell ref="E7:E10"/>
@@ -3491,36 +3524,6 @@
     <mergeCell ref="D23:D27"/>
     <mergeCell ref="B23:B42"/>
     <mergeCell ref="B52:B67"/>
-    <mergeCell ref="D49:D51"/>
-    <mergeCell ref="C49:C51"/>
-    <mergeCell ref="B43:B51"/>
-    <mergeCell ref="D43:D45"/>
-    <mergeCell ref="C43:C45"/>
-    <mergeCell ref="C46:C48"/>
-    <mergeCell ref="B3:B22"/>
-    <mergeCell ref="C3:C6"/>
-    <mergeCell ref="C7:C10"/>
-    <mergeCell ref="C11:C14"/>
-    <mergeCell ref="C15:C18"/>
-    <mergeCell ref="C19:C22"/>
-    <mergeCell ref="C23:C27"/>
-    <mergeCell ref="C28:C32"/>
-    <mergeCell ref="C33:C37"/>
-    <mergeCell ref="C38:C42"/>
-    <mergeCell ref="E46:E48"/>
-    <mergeCell ref="D38:D42"/>
-    <mergeCell ref="D28:D32"/>
-    <mergeCell ref="D46:D48"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="K6:K7"/>
-    <mergeCell ref="K10:K26"/>
-    <mergeCell ref="D19:D22"/>
-    <mergeCell ref="E3:E6"/>
-    <mergeCell ref="D3:D6"/>
-    <mergeCell ref="D15:D18"/>
-    <mergeCell ref="D7:D10"/>
-    <mergeCell ref="D11:D14"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: add 5V_An and 3V3_An
</commit_message>
<xml_diff>
--- a/ODB_V3/Hardware/Kicad/STM32F412ZGT6_Interfaces.xlsx
+++ b/ODB_V3/Hardware/Kicad/STM32F412ZGT6_Interfaces.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gagno\OneDrive\Documents\ULaval\GAUL\ODB2\Ordinateur-de-bord\ODB_V3\Hardware\Kicad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2877C714-07AB-438B-88FD-65706A253676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60D33F72-BE32-4ECE-BCC1-F36F438ADD3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="170">
   <si>
     <t>Interface</t>
   </si>
@@ -428,18 +428,6 @@
     <t>D7</t>
   </si>
   <si>
-    <t>ALE</t>
-  </si>
-  <si>
-    <t>WE#</t>
-  </si>
-  <si>
-    <t>RE#</t>
-  </si>
-  <si>
-    <t>CE#</t>
-  </si>
-  <si>
     <t>PD14</t>
   </si>
   <si>
@@ -467,51 +455,15 @@
     <t>PG6</t>
   </si>
   <si>
-    <t>NAND</t>
-  </si>
-  <si>
-    <t>I/O0</t>
-  </si>
-  <si>
-    <t>I/O1</t>
-  </si>
-  <si>
-    <t>I/O2</t>
-  </si>
-  <si>
-    <t>I/O3</t>
-  </si>
-  <si>
-    <t>I/O4</t>
-  </si>
-  <si>
-    <t>I/O5</t>
-  </si>
-  <si>
-    <t>I/O6</t>
-  </si>
-  <si>
-    <t>I/O7</t>
-  </si>
-  <si>
     <t>AF12</t>
   </si>
   <si>
-    <t>*Vérifier</t>
-  </si>
-  <si>
     <t>Push-Pull</t>
   </si>
   <si>
     <t>NWE</t>
   </si>
   <si>
-    <t>WP#</t>
-  </si>
-  <si>
-    <t>PT</t>
-  </si>
-  <si>
     <t>NOE</t>
   </si>
   <si>
@@ -530,28 +482,7 @@
     <t>NE(1234)</t>
   </si>
   <si>
-    <t>Active low</t>
-  </si>
-  <si>
-    <t>Bank select + Active low</t>
-  </si>
-  <si>
-    <t>CLW</t>
-  </si>
-  <si>
-    <t>GND / Floating</t>
-  </si>
-  <si>
-    <t>R/B#</t>
-  </si>
-  <si>
     <t>?</t>
-  </si>
-  <si>
-    <t>STM32 : p63 à 65</t>
-  </si>
-  <si>
-    <t>NAND : p12-13</t>
   </si>
   <si>
     <t>BNO055 (UART-I2C)</t>
@@ -842,7 +773,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -919,15 +850,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -940,9 +862,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -951,9 +870,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -967,31 +883,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1002,18 +924,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1418,16 +1328,16 @@
       </c>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B3" s="54" t="s">
+      <c r="B3" s="38" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="56">
+      <c r="C3" s="45">
         <v>1</v>
       </c>
-      <c r="D3" s="48" t="s">
+      <c r="D3" s="42" t="s">
         <v>90</v>
       </c>
-      <c r="E3" s="48" t="s">
+      <c r="E3" s="42" t="s">
         <v>70</v>
       </c>
       <c r="F3" s="15" t="s">
@@ -1442,7 +1352,7 @@
       <c r="I3" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="K3" s="54" t="s">
+      <c r="K3" s="38" t="s">
         <v>94</v>
       </c>
       <c r="L3" s="22" t="s">
@@ -1450,10 +1360,10 @@
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B4" s="54"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="49"/>
-      <c r="E4" s="49"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
       <c r="F4" s="2" t="s">
         <v>2</v>
       </c>
@@ -1466,16 +1376,16 @@
       <c r="I4" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="K4" s="54"/>
+      <c r="K4" s="38"/>
       <c r="L4" s="23" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="54"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="49"/>
-      <c r="E5" s="49"/>
+      <c r="B5" s="38"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
       <c r="F5" s="2" t="s">
         <v>3</v>
       </c>
@@ -1496,10 +1406,10 @@
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B6" s="54"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="49"/>
+      <c r="B6" s="38"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="43"/>
       <c r="F6" s="2" t="s">
         <v>64</v>
       </c>
@@ -1512,7 +1422,7 @@
       <c r="I6" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="K6" s="54" t="s">
+      <c r="K6" s="38" t="s">
         <v>101</v>
       </c>
       <c r="L6" s="22" t="s">
@@ -1520,14 +1430,14 @@
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B7" s="54"/>
-      <c r="C7" s="56">
+      <c r="B7" s="38"/>
+      <c r="C7" s="45">
         <v>2</v>
       </c>
-      <c r="D7" s="48" t="s">
+      <c r="D7" s="42" t="s">
         <v>91</v>
       </c>
-      <c r="E7" s="48" t="s">
+      <c r="E7" s="42" t="s">
         <v>71</v>
       </c>
       <c r="F7" s="15" t="s">
@@ -1542,16 +1452,16 @@
       <c r="I7" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="K7" s="54"/>
+      <c r="K7" s="38"/>
       <c r="L7" s="23" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B8" s="54"/>
-      <c r="C8" s="44"/>
-      <c r="D8" s="49"/>
-      <c r="E8" s="49"/>
+      <c r="B8" s="38"/>
+      <c r="C8" s="46"/>
+      <c r="D8" s="43"/>
+      <c r="E8" s="43"/>
       <c r="F8" s="2" t="s">
         <v>2</v>
       </c>
@@ -1572,10 +1482,10 @@
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B9" s="54"/>
-      <c r="C9" s="44"/>
-      <c r="D9" s="49"/>
-      <c r="E9" s="49"/>
+      <c r="B9" s="38"/>
+      <c r="C9" s="46"/>
+      <c r="D9" s="43"/>
+      <c r="E9" s="43"/>
       <c r="F9" s="2" t="s">
         <v>3</v>
       </c>
@@ -1596,10 +1506,10 @@
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B10" s="54"/>
-      <c r="C10" s="55"/>
-      <c r="D10" s="50"/>
-      <c r="E10" s="50"/>
+      <c r="B10" s="38"/>
+      <c r="C10" s="47"/>
+      <c r="D10" s="44"/>
+      <c r="E10" s="44"/>
       <c r="F10" s="9" t="s">
         <v>64</v>
       </c>
@@ -1612,19 +1522,19 @@
       <c r="I10" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="K10" s="42" t="s">
+      <c r="K10" s="39" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="54"/>
-      <c r="C11" s="56">
+      <c r="B11" s="38"/>
+      <c r="C11" s="45">
         <v>3</v>
       </c>
-      <c r="D11" s="48" t="s">
+      <c r="D11" s="42" t="s">
         <v>91</v>
       </c>
-      <c r="E11" s="48" t="s">
+      <c r="E11" s="42" t="s">
         <v>71</v>
       </c>
       <c r="F11" s="15" t="s">
@@ -1639,13 +1549,13 @@
       <c r="I11" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="K11" s="43"/>
+      <c r="K11" s="40"/>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B12" s="54"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="49"/>
-      <c r="E12" s="49"/>
+      <c r="B12" s="38"/>
+      <c r="C12" s="46"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="43"/>
       <c r="F12" s="2" t="s">
         <v>2</v>
       </c>
@@ -1658,13 +1568,13 @@
       <c r="I12" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="K12" s="43"/>
+      <c r="K12" s="40"/>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B13" s="54"/>
-      <c r="C13" s="44"/>
-      <c r="D13" s="49"/>
-      <c r="E13" s="49"/>
+      <c r="B13" s="38"/>
+      <c r="C13" s="46"/>
+      <c r="D13" s="43"/>
+      <c r="E13" s="43"/>
       <c r="F13" s="2" t="s">
         <v>3</v>
       </c>
@@ -1677,13 +1587,13 @@
       <c r="I13" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="K13" s="43"/>
+      <c r="K13" s="40"/>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B14" s="54"/>
-      <c r="C14" s="55"/>
-      <c r="D14" s="50"/>
-      <c r="E14" s="50"/>
+      <c r="B14" s="38"/>
+      <c r="C14" s="47"/>
+      <c r="D14" s="44"/>
+      <c r="E14" s="44"/>
       <c r="F14" s="9" t="s">
         <v>64</v>
       </c>
@@ -1696,17 +1606,17 @@
       <c r="I14" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="K14" s="43"/>
+      <c r="K14" s="40"/>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B15" s="54"/>
-      <c r="C15" s="56">
+      <c r="B15" s="38"/>
+      <c r="C15" s="45">
         <v>4</v>
       </c>
-      <c r="D15" s="48" t="s">
+      <c r="D15" s="42" t="s">
         <v>90</v>
       </c>
-      <c r="E15" s="48" t="s">
+      <c r="E15" s="42" t="s">
         <v>70</v>
       </c>
       <c r="F15" s="15" t="s">
@@ -1721,13 +1631,13 @@
       <c r="I15" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="K15" s="43"/>
+      <c r="K15" s="40"/>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B16" s="54"/>
-      <c r="C16" s="44"/>
-      <c r="D16" s="49"/>
-      <c r="E16" s="49"/>
+      <c r="B16" s="38"/>
+      <c r="C16" s="46"/>
+      <c r="D16" s="43"/>
+      <c r="E16" s="43"/>
       <c r="F16" s="2" t="s">
         <v>2</v>
       </c>
@@ -1740,13 +1650,13 @@
       <c r="I16" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="K16" s="43"/>
+      <c r="K16" s="40"/>
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B17" s="54"/>
-      <c r="C17" s="44"/>
-      <c r="D17" s="49"/>
-      <c r="E17" s="49"/>
+      <c r="B17" s="38"/>
+      <c r="C17" s="46"/>
+      <c r="D17" s="43"/>
+      <c r="E17" s="43"/>
       <c r="F17" s="2" t="s">
         <v>3</v>
       </c>
@@ -1759,13 +1669,13 @@
       <c r="I17" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="K17" s="43"/>
+      <c r="K17" s="40"/>
     </row>
     <row r="18" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B18" s="54"/>
-      <c r="C18" s="55"/>
-      <c r="D18" s="50"/>
-      <c r="E18" s="50"/>
+      <c r="B18" s="38"/>
+      <c r="C18" s="47"/>
+      <c r="D18" s="44"/>
+      <c r="E18" s="44"/>
       <c r="F18" s="9" t="s">
         <v>64</v>
       </c>
@@ -1778,17 +1688,17 @@
       <c r="I18" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="K18" s="43"/>
+      <c r="K18" s="40"/>
     </row>
     <row r="19" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B19" s="54"/>
-      <c r="C19" s="56">
+      <c r="B19" s="38"/>
+      <c r="C19" s="45">
         <v>5</v>
       </c>
-      <c r="D19" s="48" t="s">
+      <c r="D19" s="42" t="s">
         <v>90</v>
       </c>
-      <c r="E19" s="48" t="s">
+      <c r="E19" s="42" t="s">
         <v>70</v>
       </c>
       <c r="F19" s="15" t="s">
@@ -1803,13 +1713,13 @@
       <c r="I19" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="K19" s="43"/>
+      <c r="K19" s="40"/>
     </row>
     <row r="20" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B20" s="54"/>
-      <c r="C20" s="44"/>
-      <c r="D20" s="49"/>
-      <c r="E20" s="49"/>
+      <c r="B20" s="38"/>
+      <c r="C20" s="46"/>
+      <c r="D20" s="43"/>
+      <c r="E20" s="43"/>
       <c r="F20" s="2" t="s">
         <v>2</v>
       </c>
@@ -1822,13 +1732,13 @@
       <c r="I20" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="K20" s="43"/>
+      <c r="K20" s="40"/>
     </row>
     <row r="21" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B21" s="54"/>
-      <c r="C21" s="44"/>
-      <c r="D21" s="49"/>
-      <c r="E21" s="49"/>
+      <c r="B21" s="38"/>
+      <c r="C21" s="46"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
       <c r="F21" s="2" t="s">
         <v>3</v>
       </c>
@@ -1841,13 +1751,13 @@
       <c r="I21" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="K21" s="43"/>
+      <c r="K21" s="40"/>
     </row>
     <row r="22" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B22" s="54"/>
-      <c r="C22" s="55"/>
-      <c r="D22" s="50"/>
-      <c r="E22" s="50"/>
+      <c r="B22" s="38"/>
+      <c r="C22" s="47"/>
+      <c r="D22" s="44"/>
+      <c r="E22" s="44"/>
       <c r="F22" s="9" t="s">
         <v>64</v>
       </c>
@@ -1860,19 +1770,19 @@
       <c r="I22" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="K22" s="43"/>
+      <c r="K22" s="40"/>
     </row>
     <row r="23" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B23" s="54" t="s">
+      <c r="B23" s="38" t="s">
         <v>65</v>
       </c>
-      <c r="C23" s="56">
+      <c r="C23" s="45">
         <v>1</v>
       </c>
-      <c r="D23" s="48" t="s">
+      <c r="D23" s="42" t="s">
         <v>90</v>
       </c>
-      <c r="E23" s="48" t="s">
+      <c r="E23" s="42" t="s">
         <v>68</v>
       </c>
       <c r="F23" s="15" t="s">
@@ -1887,13 +1797,13 @@
       <c r="I23" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="K23" s="43"/>
+      <c r="K23" s="40"/>
     </row>
     <row r="24" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B24" s="54"/>
-      <c r="C24" s="44"/>
-      <c r="D24" s="49"/>
-      <c r="E24" s="49"/>
+      <c r="B24" s="38"/>
+      <c r="C24" s="46"/>
+      <c r="D24" s="43"/>
+      <c r="E24" s="43"/>
       <c r="F24" s="2" t="s">
         <v>5</v>
       </c>
@@ -1906,13 +1816,13 @@
       <c r="I24" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="K24" s="43"/>
+      <c r="K24" s="40"/>
     </row>
     <row r="25" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B25" s="54"/>
-      <c r="C25" s="44"/>
-      <c r="D25" s="49"/>
-      <c r="E25" s="49"/>
+      <c r="B25" s="38"/>
+      <c r="C25" s="46"/>
+      <c r="D25" s="43"/>
+      <c r="E25" s="43"/>
       <c r="F25" s="2" t="s">
         <v>6</v>
       </c>
@@ -1925,13 +1835,13 @@
       <c r="I25" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="K25" s="43"/>
+      <c r="K25" s="40"/>
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B26" s="54"/>
-      <c r="C26" s="44"/>
-      <c r="D26" s="49"/>
-      <c r="E26" s="49"/>
+      <c r="B26" s="38"/>
+      <c r="C26" s="46"/>
+      <c r="D26" s="43"/>
+      <c r="E26" s="43"/>
       <c r="F26" s="2" t="s">
         <v>7</v>
       </c>
@@ -1944,13 +1854,13 @@
       <c r="I26" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="K26" s="45"/>
+      <c r="K26" s="41"/>
     </row>
     <row r="27" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B27" s="54"/>
-      <c r="C27" s="44"/>
-      <c r="D27" s="49"/>
-      <c r="E27" s="49"/>
+      <c r="B27" s="38"/>
+      <c r="C27" s="46"/>
+      <c r="D27" s="43"/>
+      <c r="E27" s="43"/>
       <c r="F27" s="2" t="s">
         <v>8</v>
       </c>
@@ -1968,14 +1878,14 @@
       </c>
     </row>
     <row r="28" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B28" s="54"/>
-      <c r="C28" s="56">
+      <c r="B28" s="38"/>
+      <c r="C28" s="45">
         <v>2</v>
       </c>
-      <c r="D28" s="48" t="s">
+      <c r="D28" s="42" t="s">
         <v>91</v>
       </c>
-      <c r="E28" s="48" t="s">
+      <c r="E28" s="42" t="s">
         <v>69</v>
       </c>
       <c r="F28" s="15" t="s">
@@ -1992,10 +1902,10 @@
       </c>
     </row>
     <row r="29" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B29" s="54"/>
-      <c r="C29" s="44"/>
-      <c r="D29" s="49"/>
-      <c r="E29" s="49"/>
+      <c r="B29" s="38"/>
+      <c r="C29" s="46"/>
+      <c r="D29" s="43"/>
+      <c r="E29" s="43"/>
       <c r="F29" s="2" t="s">
         <v>5</v>
       </c>
@@ -2010,10 +1920,10 @@
       </c>
     </row>
     <row r="30" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B30" s="54"/>
-      <c r="C30" s="44"/>
-      <c r="D30" s="49"/>
-      <c r="E30" s="49"/>
+      <c r="B30" s="38"/>
+      <c r="C30" s="46"/>
+      <c r="D30" s="43"/>
+      <c r="E30" s="43"/>
       <c r="F30" s="2" t="s">
         <v>6</v>
       </c>
@@ -2028,10 +1938,10 @@
       </c>
     </row>
     <row r="31" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B31" s="54"/>
-      <c r="C31" s="44"/>
-      <c r="D31" s="49"/>
-      <c r="E31" s="49"/>
+      <c r="B31" s="38"/>
+      <c r="C31" s="46"/>
+      <c r="D31" s="43"/>
+      <c r="E31" s="43"/>
       <c r="F31" s="2" t="s">
         <v>7</v>
       </c>
@@ -2046,10 +1956,10 @@
       </c>
     </row>
     <row r="32" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B32" s="54"/>
-      <c r="C32" s="55"/>
-      <c r="D32" s="50"/>
-      <c r="E32" s="50"/>
+      <c r="B32" s="38"/>
+      <c r="C32" s="47"/>
+      <c r="D32" s="44"/>
+      <c r="E32" s="44"/>
       <c r="F32" s="9" t="s">
         <v>8</v>
       </c>
@@ -2064,14 +1974,14 @@
       </c>
     </row>
     <row r="33" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B33" s="54"/>
-      <c r="C33" s="56">
+      <c r="B33" s="38"/>
+      <c r="C33" s="45">
         <v>3</v>
       </c>
-      <c r="D33" s="48" t="s">
+      <c r="D33" s="42" t="s">
         <v>91</v>
       </c>
-      <c r="E33" s="48" t="s">
+      <c r="E33" s="42" t="s">
         <v>69</v>
       </c>
       <c r="F33" s="15" t="s">
@@ -2086,20 +1996,20 @@
       <c r="I33" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="K33" s="57" t="s">
+      <c r="K33" s="37" t="s">
         <v>112</v>
       </c>
-      <c r="L33" s="57"/>
+      <c r="L33" s="37"/>
       <c r="M33" s="1" t="s">
-        <v>186</v>
+        <v>163</v>
       </c>
       <c r="N33" s="1"/>
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B34" s="54"/>
-      <c r="C34" s="44"/>
-      <c r="D34" s="49"/>
-      <c r="E34" s="49"/>
+      <c r="B34" s="38"/>
+      <c r="C34" s="46"/>
+      <c r="D34" s="43"/>
+      <c r="E34" s="43"/>
       <c r="F34" s="2" t="s">
         <v>5</v>
       </c>
@@ -2112,21 +2022,21 @@
       <c r="I34" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="K34" s="41" t="s">
-        <v>173</v>
-      </c>
-      <c r="L34" s="41" t="s">
-        <v>181</v>
-      </c>
-      <c r="M34" s="41" t="s">
-        <v>189</v>
+      <c r="K34" s="36" t="s">
+        <v>150</v>
+      </c>
+      <c r="L34" s="36" t="s">
+        <v>158</v>
+      </c>
+      <c r="M34" s="36" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="35" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B35" s="54"/>
-      <c r="C35" s="44"/>
-      <c r="D35" s="49"/>
-      <c r="E35" s="49"/>
+      <c r="B35" s="38"/>
+      <c r="C35" s="46"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="43"/>
       <c r="F35" s="2" t="s">
         <v>6</v>
       </c>
@@ -2139,21 +2049,21 @@
       <c r="I35" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="K35" s="41" t="s">
-        <v>175</v>
-      </c>
-      <c r="L35" s="41" t="s">
-        <v>191</v>
-      </c>
-      <c r="M35" s="41" t="s">
-        <v>187</v>
+      <c r="K35" s="36" t="s">
+        <v>152</v>
+      </c>
+      <c r="L35" s="36" t="s">
+        <v>168</v>
+      </c>
+      <c r="M35" s="36" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="36" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B36" s="54"/>
-      <c r="C36" s="44"/>
-      <c r="D36" s="49"/>
-      <c r="E36" s="49"/>
+      <c r="B36" s="38"/>
+      <c r="C36" s="46"/>
+      <c r="D36" s="43"/>
+      <c r="E36" s="43"/>
       <c r="F36" s="2" t="s">
         <v>7</v>
       </c>
@@ -2166,21 +2076,21 @@
       <c r="I36" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="K36" s="41" t="s">
-        <v>180</v>
-      </c>
-      <c r="L36" s="41" t="s">
-        <v>183</v>
-      </c>
-      <c r="M36" s="41" t="s">
-        <v>189</v>
+      <c r="K36" s="36" t="s">
+        <v>157</v>
+      </c>
+      <c r="L36" s="36" t="s">
+        <v>160</v>
+      </c>
+      <c r="M36" s="36" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B37" s="54"/>
-      <c r="C37" s="55"/>
-      <c r="D37" s="50"/>
-      <c r="E37" s="50"/>
+      <c r="B37" s="38"/>
+      <c r="C37" s="47"/>
+      <c r="D37" s="44"/>
+      <c r="E37" s="44"/>
       <c r="F37" s="9" t="s">
         <v>8</v>
       </c>
@@ -2193,25 +2103,25 @@
       <c r="I37" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="K37" s="41" t="s">
+      <c r="K37" s="36" t="s">
         <v>114</v>
       </c>
-      <c r="L37" s="41" t="s">
-        <v>182</v>
-      </c>
-      <c r="M37" s="41" t="s">
+      <c r="L37" s="36" t="s">
+        <v>159</v>
+      </c>
+      <c r="M37" s="36" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B38" s="54"/>
-      <c r="C38" s="56">
+      <c r="B38" s="38"/>
+      <c r="C38" s="45">
         <v>6</v>
       </c>
-      <c r="D38" s="48" t="s">
+      <c r="D38" s="42" t="s">
         <v>90</v>
       </c>
-      <c r="E38" s="48" t="s">
+      <c r="E38" s="42" t="s">
         <v>68</v>
       </c>
       <c r="F38" s="15" t="s">
@@ -2226,21 +2136,21 @@
       <c r="I38" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="K38" s="41" t="s">
+      <c r="K38" s="36" t="s">
         <v>113</v>
       </c>
-      <c r="L38" s="41" t="s">
-        <v>179</v>
-      </c>
-      <c r="M38" s="41" t="s">
-        <v>190</v>
+      <c r="L38" s="36" t="s">
+        <v>156</v>
+      </c>
+      <c r="M38" s="36" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="39" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B39" s="54"/>
-      <c r="C39" s="44"/>
-      <c r="D39" s="49"/>
-      <c r="E39" s="49"/>
+      <c r="B39" s="38"/>
+      <c r="C39" s="46"/>
+      <c r="D39" s="43"/>
+      <c r="E39" s="43"/>
       <c r="F39" s="2" t="s">
         <v>5</v>
       </c>
@@ -2253,21 +2163,21 @@
       <c r="I39" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="K39" s="41" t="s">
+      <c r="K39" s="36" t="s">
         <v>115</v>
       </c>
-      <c r="L39" s="41" t="s">
-        <v>177</v>
-      </c>
-      <c r="M39" s="41" t="s">
-        <v>190</v>
+      <c r="L39" s="36" t="s">
+        <v>154</v>
+      </c>
+      <c r="M39" s="36" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B40" s="54"/>
-      <c r="C40" s="44"/>
-      <c r="D40" s="49"/>
-      <c r="E40" s="49"/>
+      <c r="B40" s="38"/>
+      <c r="C40" s="46"/>
+      <c r="D40" s="43"/>
+      <c r="E40" s="43"/>
       <c r="F40" s="2" t="s">
         <v>6</v>
       </c>
@@ -2280,21 +2190,21 @@
       <c r="I40" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="K40" s="41" t="s">
-        <v>174</v>
-      </c>
-      <c r="L40" s="41" t="s">
-        <v>192</v>
-      </c>
-      <c r="M40" s="41" t="s">
+      <c r="K40" s="36" t="s">
+        <v>151</v>
+      </c>
+      <c r="L40" s="36" t="s">
+        <v>169</v>
+      </c>
+      <c r="M40" s="36" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B41" s="54"/>
-      <c r="C41" s="44"/>
-      <c r="D41" s="49"/>
-      <c r="E41" s="49"/>
+      <c r="B41" s="38"/>
+      <c r="C41" s="46"/>
+      <c r="D41" s="43"/>
+      <c r="E41" s="43"/>
       <c r="F41" s="2" t="s">
         <v>7</v>
       </c>
@@ -2307,21 +2217,21 @@
       <c r="I41" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="K41" s="41" t="s">
-        <v>178</v>
-      </c>
-      <c r="L41" s="41" t="s">
-        <v>185</v>
-      </c>
-      <c r="M41" s="41" t="s">
+      <c r="K41" s="36" t="s">
+        <v>155</v>
+      </c>
+      <c r="L41" s="36" t="s">
+        <v>162</v>
+      </c>
+      <c r="M41" s="36" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B42" s="54"/>
-      <c r="C42" s="55"/>
-      <c r="D42" s="50"/>
-      <c r="E42" s="50"/>
+      <c r="B42" s="38"/>
+      <c r="C42" s="47"/>
+      <c r="D42" s="44"/>
+      <c r="E42" s="44"/>
       <c r="F42" s="9" t="s">
         <v>8</v>
       </c>
@@ -2334,27 +2244,27 @@
       <c r="I42" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="K42" s="41" t="s">
-        <v>176</v>
-      </c>
-      <c r="L42" s="41" t="s">
-        <v>184</v>
-      </c>
-      <c r="M42" s="41" t="s">
-        <v>188</v>
+      <c r="K42" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="L42" s="36" t="s">
+        <v>161</v>
+      </c>
+      <c r="M42" s="36" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="43" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B43" s="54" t="s">
+      <c r="B43" s="38" t="s">
         <v>66</v>
       </c>
-      <c r="C43" s="56">
+      <c r="C43" s="45">
         <v>1</v>
       </c>
-      <c r="D43" s="48" t="s">
+      <c r="D43" s="42" t="s">
         <v>91</v>
       </c>
-      <c r="E43" s="51" t="s">
+      <c r="E43" s="48" t="s">
         <v>92</v>
       </c>
       <c r="F43" s="15" t="s">
@@ -2371,10 +2281,10 @@
       </c>
     </row>
     <row r="44" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B44" s="54"/>
-      <c r="C44" s="44"/>
-      <c r="D44" s="49"/>
-      <c r="E44" s="52"/>
+      <c r="B44" s="38"/>
+      <c r="C44" s="46"/>
+      <c r="D44" s="43"/>
+      <c r="E44" s="49"/>
       <c r="F44" s="2" t="s">
         <v>10</v>
       </c>
@@ -2389,10 +2299,10 @@
       </c>
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B45" s="54"/>
-      <c r="C45" s="55"/>
-      <c r="D45" s="50"/>
-      <c r="E45" s="53"/>
+      <c r="B45" s="38"/>
+      <c r="C45" s="47"/>
+      <c r="D45" s="44"/>
+      <c r="E45" s="50"/>
       <c r="F45" s="9" t="s">
         <v>11</v>
       </c>
@@ -2407,14 +2317,14 @@
       </c>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B46" s="54"/>
-      <c r="C46" s="56">
+      <c r="B46" s="38"/>
+      <c r="C46" s="45">
         <v>2</v>
       </c>
-      <c r="D46" s="48" t="s">
+      <c r="D46" s="42" t="s">
         <v>91</v>
       </c>
-      <c r="E46" s="48" t="s">
+      <c r="E46" s="42" t="s">
         <v>67</v>
       </c>
       <c r="F46" s="15" t="s">
@@ -2431,10 +2341,10 @@
       </c>
     </row>
     <row r="47" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B47" s="54"/>
-      <c r="C47" s="44"/>
-      <c r="D47" s="49"/>
-      <c r="E47" s="49"/>
+      <c r="B47" s="38"/>
+      <c r="C47" s="46"/>
+      <c r="D47" s="43"/>
+      <c r="E47" s="43"/>
       <c r="F47" s="2" t="s">
         <v>10</v>
       </c>
@@ -2449,10 +2359,10 @@
       </c>
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B48" s="54"/>
-      <c r="C48" s="55"/>
-      <c r="D48" s="50"/>
-      <c r="E48" s="50"/>
+      <c r="B48" s="38"/>
+      <c r="C48" s="47"/>
+      <c r="D48" s="44"/>
+      <c r="E48" s="44"/>
       <c r="F48" s="9" t="s">
         <v>11</v>
       </c>
@@ -2467,14 +2377,14 @@
       </c>
     </row>
     <row r="49" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B49" s="54"/>
-      <c r="C49" s="44">
+      <c r="B49" s="38"/>
+      <c r="C49" s="46">
         <v>3</v>
       </c>
-      <c r="D49" s="49" t="s">
+      <c r="D49" s="43" t="s">
         <v>91</v>
       </c>
-      <c r="E49" s="49" t="s">
+      <c r="E49" s="43" t="s">
         <v>67</v>
       </c>
       <c r="F49" s="2" t="s">
@@ -2491,10 +2401,10 @@
       </c>
     </row>
     <row r="50" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B50" s="54"/>
-      <c r="C50" s="44"/>
-      <c r="D50" s="49"/>
-      <c r="E50" s="49"/>
+      <c r="B50" s="38"/>
+      <c r="C50" s="46"/>
+      <c r="D50" s="43"/>
+      <c r="E50" s="43"/>
       <c r="F50" s="2" t="s">
         <v>10</v>
       </c>
@@ -2509,10 +2419,10 @@
       </c>
     </row>
     <row r="51" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B51" s="54"/>
-      <c r="C51" s="55"/>
-      <c r="D51" s="50"/>
-      <c r="E51" s="50"/>
+      <c r="B51" s="38"/>
+      <c r="C51" s="47"/>
+      <c r="D51" s="44"/>
+      <c r="E51" s="44"/>
       <c r="F51" s="9" t="s">
         <v>11</v>
       </c>
@@ -2527,7 +2437,7 @@
       </c>
     </row>
     <row r="52" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B52" s="54" t="s">
+      <c r="B52" s="38" t="s">
         <v>83</v>
       </c>
       <c r="C52" s="18">
@@ -2555,7 +2465,7 @@
       </c>
     </row>
     <row r="53" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B53" s="54"/>
+      <c r="B53" s="38"/>
       <c r="C53" s="19">
         <v>1</v>
       </c>
@@ -2581,7 +2491,7 @@
       </c>
     </row>
     <row r="54" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B54" s="54"/>
+      <c r="B54" s="38"/>
       <c r="C54" s="19">
         <v>2</v>
       </c>
@@ -2607,7 +2517,7 @@
       </c>
     </row>
     <row r="55" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B55" s="54"/>
+      <c r="B55" s="38"/>
       <c r="C55" s="19">
         <v>3</v>
       </c>
@@ -2633,7 +2543,7 @@
       </c>
     </row>
     <row r="56" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B56" s="54"/>
+      <c r="B56" s="38"/>
       <c r="C56" s="19">
         <v>4</v>
       </c>
@@ -2659,7 +2569,7 @@
       </c>
     </row>
     <row r="57" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B57" s="54"/>
+      <c r="B57" s="38"/>
       <c r="C57" s="19">
         <v>5</v>
       </c>
@@ -2685,7 +2595,7 @@
       </c>
     </row>
     <row r="58" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B58" s="54"/>
+      <c r="B58" s="38"/>
       <c r="C58" s="19">
         <v>6</v>
       </c>
@@ -2711,7 +2621,7 @@
       </c>
     </row>
     <row r="59" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B59" s="54"/>
+      <c r="B59" s="38"/>
       <c r="C59" s="19">
         <v>7</v>
       </c>
@@ -2737,7 +2647,7 @@
       </c>
     </row>
     <row r="60" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B60" s="54"/>
+      <c r="B60" s="38"/>
       <c r="C60" s="19">
         <v>8</v>
       </c>
@@ -2763,7 +2673,7 @@
       </c>
     </row>
     <row r="61" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B61" s="54"/>
+      <c r="B61" s="38"/>
       <c r="C61" s="19">
         <v>9</v>
       </c>
@@ -2789,7 +2699,7 @@
       </c>
     </row>
     <row r="62" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B62" s="54"/>
+      <c r="B62" s="38"/>
       <c r="C62" s="19">
         <v>10</v>
       </c>
@@ -2815,7 +2725,7 @@
       </c>
     </row>
     <row r="63" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B63" s="54"/>
+      <c r="B63" s="38"/>
       <c r="C63" s="19">
         <v>11</v>
       </c>
@@ -2844,7 +2754,7 @@
       </c>
     </row>
     <row r="64" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B64" s="54"/>
+      <c r="B64" s="38"/>
       <c r="C64" s="19">
         <v>12</v>
       </c>
@@ -2873,7 +2783,7 @@
       </c>
     </row>
     <row r="65" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B65" s="54"/>
+      <c r="B65" s="38"/>
       <c r="C65" s="19">
         <v>13</v>
       </c>
@@ -2899,7 +2809,7 @@
       </c>
     </row>
     <row r="66" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B66" s="54"/>
+      <c r="B66" s="38"/>
       <c r="C66" s="19">
         <v>14</v>
       </c>
@@ -2925,7 +2835,7 @@
       </c>
     </row>
     <row r="67" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B67" s="54"/>
+      <c r="B67" s="38"/>
       <c r="C67" s="20">
         <v>15</v>
       </c>
@@ -2949,13 +2859,11 @@
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
-      <c r="J67" s="46" t="s">
-        <v>144</v>
-      </c>
-      <c r="K67" s="47"/>
+      <c r="J67"/>
+      <c r="K67"/>
     </row>
     <row r="68" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B68" s="42" t="s">
+      <c r="B68" s="39" t="s">
         <v>94</v>
       </c>
       <c r="C68" s="14" t="s">
@@ -2973,21 +2881,19 @@
         <v>116</v>
       </c>
       <c r="G68" s="15" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="H68" s="15" t="s">
         <v>87</v>
       </c>
       <c r="I68" s="16" t="s">
-        <v>153</v>
-      </c>
-      <c r="J68" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="K68" s="26"/>
+        <v>140</v>
+      </c>
+      <c r="J68"/>
+      <c r="K68"/>
     </row>
     <row r="69" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B69" s="43"/>
+      <c r="B69" s="40"/>
       <c r="C69" s="6" t="s">
         <v>124</v>
       </c>
@@ -3003,21 +2909,19 @@
         <v>116</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="H69" s="2" t="s">
         <v>87</v>
       </c>
       <c r="I69" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="J69" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="K69" s="26"/>
+        <v>140</v>
+      </c>
+      <c r="J69"/>
+      <c r="K69"/>
     </row>
     <row r="70" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B70" s="43"/>
+      <c r="B70" s="40"/>
       <c r="C70" s="6" t="s">
         <v>125</v>
       </c>
@@ -3033,21 +2937,19 @@
         <v>116</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="H70" s="2" t="s">
         <v>87</v>
       </c>
       <c r="I70" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="J70" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="K70" s="26"/>
+        <v>140</v>
+      </c>
+      <c r="J70"/>
+      <c r="K70"/>
     </row>
     <row r="71" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B71" s="43"/>
+      <c r="B71" s="40"/>
       <c r="C71" s="6" t="s">
         <v>126</v>
       </c>
@@ -3063,21 +2965,19 @@
         <v>116</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="H71" s="2" t="s">
         <v>87</v>
       </c>
       <c r="I71" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="J71" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="K71" s="26"/>
+        <v>140</v>
+      </c>
+      <c r="J71"/>
+      <c r="K71"/>
     </row>
     <row r="72" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B72" s="43"/>
+      <c r="B72" s="40"/>
       <c r="C72" s="6" t="s">
         <v>127</v>
       </c>
@@ -3093,21 +2993,19 @@
         <v>116</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="H72" s="2" t="s">
         <v>87</v>
       </c>
       <c r="I72" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="J72" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="K72" s="26"/>
+        <v>140</v>
+      </c>
+      <c r="J72"/>
+      <c r="K72"/>
     </row>
     <row r="73" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B73" s="43"/>
+      <c r="B73" s="40"/>
       <c r="C73" s="6" t="s">
         <v>128</v>
       </c>
@@ -3123,21 +3021,19 @@
         <v>116</v>
       </c>
       <c r="G73" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="H73" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="I73" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="H73" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="I73" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="J73" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="K73" s="26"/>
+      <c r="J73"/>
+      <c r="K73"/>
     </row>
     <row r="74" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B74" s="43"/>
+      <c r="B74" s="40"/>
       <c r="C74" s="6" t="s">
         <v>129</v>
       </c>
@@ -3153,21 +3049,19 @@
         <v>116</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="H74" s="2" t="s">
         <v>87</v>
       </c>
       <c r="I74" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="J74" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="K74" s="26"/>
+        <v>140</v>
+      </c>
+      <c r="J74"/>
+      <c r="K74"/>
     </row>
     <row r="75" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B75" s="43"/>
+      <c r="B75" s="40"/>
       <c r="C75" s="6" t="s">
         <v>130</v>
       </c>
@@ -3183,23 +3077,21 @@
         <v>116</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="H75" s="2" t="s">
         <v>87</v>
       </c>
       <c r="I75" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="J75" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="K75" s="26"/>
+        <v>140</v>
+      </c>
+      <c r="J75"/>
+      <c r="K75"/>
     </row>
     <row r="76" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B76" s="43"/>
-      <c r="C76" s="29" t="s">
-        <v>170</v>
+      <c r="B76" s="40"/>
+      <c r="C76" s="26" t="s">
+        <v>149</v>
       </c>
       <c r="D76" s="2" t="str">
         <f t="shared" si="2"/>
@@ -3219,19 +3111,15 @@
         <v>87</v>
       </c>
       <c r="I76" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="J76" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="K76" s="27" t="s">
-        <v>154</v>
-      </c>
+        <v>140</v>
+      </c>
+      <c r="J76"/>
+      <c r="K76"/>
     </row>
     <row r="77" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B77" s="43"/>
-      <c r="C77" s="29" t="s">
-        <v>170</v>
+      <c r="B77" s="40"/>
+      <c r="C77" s="26" t="s">
+        <v>149</v>
       </c>
       <c r="D77" s="2" t="str">
         <f t="shared" si="2"/>
@@ -3251,19 +3139,15 @@
         <v>87</v>
       </c>
       <c r="I77" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="J77" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="K77" s="27" t="s">
-        <v>154</v>
-      </c>
+        <v>140</v>
+      </c>
+      <c r="J77"/>
+      <c r="K77"/>
     </row>
     <row r="78" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B78" s="43"/>
+      <c r="B78" s="40"/>
       <c r="C78" s="6" t="s">
-        <v>156</v>
+        <v>142</v>
       </c>
       <c r="D78" s="2" t="str">
         <f t="shared" si="2"/>
@@ -3283,19 +3167,15 @@
         <v>87</v>
       </c>
       <c r="I78" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="J78" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="K78" s="26" t="s">
-        <v>165</v>
-      </c>
+        <v>140</v>
+      </c>
+      <c r="J78"/>
+      <c r="K78"/>
     </row>
     <row r="79" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B79" s="43"/>
+      <c r="B79" s="40"/>
       <c r="C79" s="6" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="D79" s="2" t="str">
         <f t="shared" si="2"/>
@@ -3315,51 +3195,43 @@
         <v>87</v>
       </c>
       <c r="I79" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="J79" s="28" t="s">
-        <v>133</v>
-      </c>
-      <c r="K79" s="26" t="s">
-        <v>166</v>
-      </c>
+        <v>140</v>
+      </c>
+      <c r="J79"/>
+      <c r="K79"/>
     </row>
     <row r="80" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B80" s="43"/>
-      <c r="C80" s="29" t="s">
-        <v>164</v>
-      </c>
-      <c r="D80" s="30" t="str">
+      <c r="B80" s="40"/>
+      <c r="C80" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="D80" s="27" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E80" s="30" t="str">
+      <c r="E80" s="27" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="F80" s="31" t="s">
+      <c r="F80" s="28" t="s">
         <v>121</v>
       </c>
-      <c r="G80" s="30" t="s">
+      <c r="G80" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="H80" s="30" t="s">
-        <v>87</v>
-      </c>
-      <c r="I80" s="32" t="s">
-        <v>153</v>
-      </c>
-      <c r="J80" s="29" t="s">
-        <v>134</v>
-      </c>
-      <c r="K80" s="33" t="s">
-        <v>165</v>
-      </c>
+      <c r="H80" s="27" t="s">
+        <v>87</v>
+      </c>
+      <c r="I80" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="J80"/>
+      <c r="K80"/>
     </row>
     <row r="81" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B81" s="43"/>
+      <c r="B81" s="40"/>
       <c r="C81" s="6" t="s">
-        <v>161</v>
+        <v>145</v>
       </c>
       <c r="D81" s="2" t="str">
         <f t="shared" si="2"/>
@@ -3373,99 +3245,84 @@
         <v>122</v>
       </c>
       <c r="G81" s="2" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="H81" s="2" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="I81" s="7" t="str">
         <f t="shared" ref="I81" si="3">"-"</f>
         <v>-</v>
       </c>
-      <c r="J81" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="K81" s="27" t="s">
-        <v>154</v>
-      </c>
+      <c r="J81"/>
+      <c r="K81"/>
     </row>
     <row r="82" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B82" s="43"/>
-      <c r="C82" s="34"/>
-      <c r="D82" s="35"/>
-      <c r="E82" s="35"/>
-      <c r="F82" s="35"/>
-      <c r="G82" s="35"/>
-      <c r="H82" s="35"/>
-      <c r="I82" s="36"/>
-      <c r="J82" s="34"/>
-      <c r="K82" s="36"/>
+      <c r="B82" s="40"/>
+      <c r="C82" s="30"/>
+      <c r="D82" s="31"/>
+      <c r="E82" s="31"/>
+      <c r="F82" s="31"/>
+      <c r="G82" s="31"/>
+      <c r="H82" s="31"/>
+      <c r="I82" s="32"/>
+      <c r="J82"/>
+      <c r="K82"/>
     </row>
     <row r="83" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B83" s="43"/>
+      <c r="B83" s="40"/>
       <c r="D83" s="15"/>
       <c r="E83" s="15"/>
       <c r="F83" s="15"/>
       <c r="G83" s="15"/>
       <c r="H83" s="15"/>
       <c r="I83" s="16"/>
-      <c r="K83" s="7"/>
+      <c r="J83"/>
+      <c r="K83"/>
     </row>
     <row r="84" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B84" s="44"/>
-      <c r="C84" s="29" t="s">
-        <v>160</v>
-      </c>
-      <c r="D84" s="30"/>
-      <c r="E84" s="30"/>
-      <c r="F84" s="30"/>
-      <c r="G84" s="30"/>
-      <c r="H84" s="30"/>
-      <c r="I84" s="32"/>
-      <c r="J84" s="37" t="s">
-        <v>157</v>
-      </c>
-      <c r="K84" s="33" t="s">
-        <v>165</v>
-      </c>
+      <c r="B84" s="46"/>
+      <c r="C84" s="26" t="s">
+        <v>144</v>
+      </c>
+      <c r="D84" s="27"/>
+      <c r="E84" s="27"/>
+      <c r="F84" s="27"/>
+      <c r="G84" s="27"/>
+      <c r="H84" s="27"/>
+      <c r="I84" s="29"/>
+      <c r="J84"/>
+      <c r="K84"/>
     </row>
     <row r="85" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B85" s="43"/>
-      <c r="C85" s="29" t="s">
-        <v>162</v>
-      </c>
-      <c r="D85" s="30"/>
-      <c r="E85" s="30"/>
-      <c r="F85" s="30"/>
-      <c r="G85" s="30"/>
-      <c r="H85" s="30"/>
-      <c r="I85" s="32"/>
-      <c r="J85" s="29" t="s">
-        <v>158</v>
-      </c>
-      <c r="K85" s="33" t="s">
-        <v>168</v>
-      </c>
-      <c r="L85" s="1" t="s">
-        <v>171</v>
-      </c>
+      <c r="B85" s="40"/>
+      <c r="C85" s="26" t="s">
+        <v>146</v>
+      </c>
+      <c r="D85" s="27"/>
+      <c r="E85" s="27"/>
+      <c r="F85" s="27"/>
+      <c r="G85" s="27"/>
+      <c r="H85" s="27"/>
+      <c r="I85" s="29"/>
+      <c r="J85"/>
+      <c r="K85"/>
+      <c r="L85" s="1"/>
     </row>
     <row r="86" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B86" s="45"/>
-      <c r="C86" s="38" t="s">
-        <v>163</v>
-      </c>
-      <c r="D86" s="39"/>
-      <c r="E86" s="39"/>
-      <c r="F86" s="39"/>
-      <c r="G86" s="39"/>
-      <c r="H86" s="39"/>
-      <c r="I86" s="40"/>
-      <c r="J86" s="38"/>
-      <c r="K86" s="40"/>
-      <c r="L86" s="1" t="s">
-        <v>172</v>
-      </c>
+      <c r="B86" s="41"/>
+      <c r="C86" s="33" t="s">
+        <v>147</v>
+      </c>
+      <c r="D86" s="34"/>
+      <c r="E86" s="34"/>
+      <c r="F86" s="34"/>
+      <c r="G86" s="34"/>
+      <c r="H86" s="34"/>
+      <c r="I86" s="35"/>
+      <c r="J86"/>
+      <c r="K86"/>
+      <c r="L86" s="1"/>
     </row>
     <row r="87" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B87" s="24"/>
@@ -3477,39 +3334,8 @@
       <c r="B89" s="24"/>
     </row>
   </sheetData>
-  <mergeCells count="46">
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="K6:K7"/>
-    <mergeCell ref="K10:K26"/>
-    <mergeCell ref="D19:D22"/>
-    <mergeCell ref="E3:E6"/>
-    <mergeCell ref="D3:D6"/>
-    <mergeCell ref="D15:D18"/>
-    <mergeCell ref="D7:D10"/>
-    <mergeCell ref="D11:D14"/>
-    <mergeCell ref="C23:C27"/>
-    <mergeCell ref="C28:C32"/>
-    <mergeCell ref="C33:C37"/>
-    <mergeCell ref="C38:C42"/>
-    <mergeCell ref="E46:E48"/>
-    <mergeCell ref="D38:D42"/>
-    <mergeCell ref="D28:D32"/>
-    <mergeCell ref="D46:D48"/>
-    <mergeCell ref="B3:B22"/>
-    <mergeCell ref="C3:C6"/>
-    <mergeCell ref="C7:C10"/>
-    <mergeCell ref="C11:C14"/>
-    <mergeCell ref="C15:C18"/>
-    <mergeCell ref="C19:C22"/>
-    <mergeCell ref="D49:D51"/>
-    <mergeCell ref="C49:C51"/>
-    <mergeCell ref="B43:B51"/>
-    <mergeCell ref="D43:D45"/>
-    <mergeCell ref="C43:C45"/>
-    <mergeCell ref="C46:C48"/>
+  <mergeCells count="45">
     <mergeCell ref="B68:B86"/>
-    <mergeCell ref="J67:K67"/>
     <mergeCell ref="E7:E10"/>
     <mergeCell ref="E11:E14"/>
     <mergeCell ref="E15:E18"/>
@@ -3524,6 +3350,36 @@
     <mergeCell ref="D23:D27"/>
     <mergeCell ref="B23:B42"/>
     <mergeCell ref="B52:B67"/>
+    <mergeCell ref="D49:D51"/>
+    <mergeCell ref="C49:C51"/>
+    <mergeCell ref="B43:B51"/>
+    <mergeCell ref="D43:D45"/>
+    <mergeCell ref="C43:C45"/>
+    <mergeCell ref="C46:C48"/>
+    <mergeCell ref="B3:B22"/>
+    <mergeCell ref="C3:C6"/>
+    <mergeCell ref="C7:C10"/>
+    <mergeCell ref="C11:C14"/>
+    <mergeCell ref="C15:C18"/>
+    <mergeCell ref="C19:C22"/>
+    <mergeCell ref="C23:C27"/>
+    <mergeCell ref="C28:C32"/>
+    <mergeCell ref="C33:C37"/>
+    <mergeCell ref="C38:C42"/>
+    <mergeCell ref="E46:E48"/>
+    <mergeCell ref="D38:D42"/>
+    <mergeCell ref="D28:D32"/>
+    <mergeCell ref="D46:D48"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="K6:K7"/>
+    <mergeCell ref="K10:K26"/>
+    <mergeCell ref="D19:D22"/>
+    <mergeCell ref="E3:E6"/>
+    <mergeCell ref="D3:D6"/>
+    <mergeCell ref="D15:D18"/>
+    <mergeCell ref="D7:D10"/>
+    <mergeCell ref="D11:D14"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: add all missing pins on stm32cubeide and kicad + add extend connectivities (UART3, SPI2)
Missing Pinout:
IMU_INT
TEMP_OUT
GPS_FUNCT_X
BUZZER_PWM
VIN_An
Senses_X
Fire_X
Pyro_Arm
PA_An
5V_An
3V3_An
</commit_message>
<xml_diff>
--- a/ODB_V3/Hardware/Kicad/STM32F412ZGT6_Interfaces.xlsx
+++ b/ODB_V3/Hardware/Kicad/STM32F412ZGT6_Interfaces.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gagno\OneDrive\Documents\ULaval\GAUL\ODB2\Ordinateur-de-bord\ODB_V3\Hardware\Kicad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60D33F72-BE32-4ECE-BCC1-F36F438ADD3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD43555B-939F-4972-9919-6EC1FF243058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="214">
   <si>
     <t>Interface</t>
   </si>
@@ -374,9 +374,6 @@
     <t>Interfaces Composants</t>
   </si>
   <si>
-    <t>HM-10 (UART)</t>
-  </si>
-  <si>
     <t>MS5803 (SPI)</t>
   </si>
   <si>
@@ -543,6 +540,141 @@
   </si>
   <si>
     <t>QuadSPI</t>
+  </si>
+  <si>
+    <t>MAX6612MXK</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>HM-11 (UART)</t>
+  </si>
+  <si>
+    <t>SMTB-0927-TW-R</t>
+  </si>
+  <si>
+    <t>Alimentation Vin</t>
+  </si>
+  <si>
+    <t>Alimentation 5V</t>
+  </si>
+  <si>
+    <t>Alimentation 3V3</t>
+  </si>
+  <si>
+    <t>Continuité Pyro1</t>
+  </si>
+  <si>
+    <t>Continuité Pyro2</t>
+  </si>
+  <si>
+    <t>Continuité Pyro3</t>
+  </si>
+  <si>
+    <t>Continuité Pyro4</t>
+  </si>
+  <si>
+    <t>Continuité Pyros armé</t>
+  </si>
+  <si>
+    <t>TIM10</t>
+  </si>
+  <si>
+    <t>TIM11</t>
+  </si>
+  <si>
+    <t>TIM13</t>
+  </si>
+  <si>
+    <t>TIM14</t>
+  </si>
+  <si>
+    <t>PA8,..,PA11</t>
+  </si>
+  <si>
+    <t>TIM1 - 4 channels</t>
+  </si>
+  <si>
+    <t>TIM2 - 4 channel</t>
+  </si>
+  <si>
+    <t>TIM3 - 4 chhanels</t>
+  </si>
+  <si>
+    <t>TIM4 - 4 chhanels</t>
+  </si>
+  <si>
+    <t>TIM5 - 4 chhanels</t>
+  </si>
+  <si>
+    <t>TIM8 - 4 chhanels</t>
+  </si>
+  <si>
+    <t>TIM9 - 2 chhanels</t>
+  </si>
+  <si>
+    <t>TIM12 - 2 chhanels</t>
+  </si>
+  <si>
+    <t>PA0,…,PA3</t>
+  </si>
+  <si>
+    <t>PC6,…,PC9</t>
+  </si>
+  <si>
+    <t>PB6,…, PB9</t>
+  </si>
+  <si>
+    <t>PA2, PA3</t>
+  </si>
+  <si>
+    <t>PB8</t>
+  </si>
+  <si>
+    <t>PB9</t>
+  </si>
+  <si>
+    <t>PB14,PB15</t>
+  </si>
+  <si>
+    <t>I2C3</t>
+  </si>
+  <si>
+    <t>EXTEND</t>
+  </si>
+  <si>
+    <t>SPI2</t>
+  </si>
+  <si>
+    <t>ADC - Channel10</t>
+  </si>
+  <si>
+    <t>TIM4 - Channel1</t>
+  </si>
+  <si>
+    <t>ADC - Channel11</t>
+  </si>
+  <si>
+    <t>ADC - Channel12</t>
+  </si>
+  <si>
+    <t>ADC - Channel13</t>
+  </si>
+  <si>
+    <t>ADC - Channel0</t>
+  </si>
+  <si>
+    <t>ADC - Channel1</t>
+  </si>
+  <si>
+    <t>ADC - Channel4</t>
+  </si>
+  <si>
+    <t>ADC - Channel5</t>
+  </si>
+  <si>
+    <t>ADC - Channel8</t>
   </si>
 </sst>
 </file>
@@ -773,7 +905,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -787,9 +919,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -841,9 +970,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -883,10 +1009,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
@@ -895,6 +1018,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -905,15 +1031,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -924,6 +1041,44 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -946,16 +1101,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>35876</xdr:colOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>55583</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>32540</xdr:rowOff>
+      <xdr:rowOff>45678</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>815682</xdr:colOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>178492</xdr:colOff>
       <xdr:row>25</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
+      <xdr:rowOff>184588</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -978,8 +1133,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8579801" y="1747040"/>
-          <a:ext cx="3365477" cy="3186910"/>
+          <a:off x="11492152" y="1760178"/>
+          <a:ext cx="3361409" cy="3186910"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1278,7 +1433,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:N89"/>
+  <dimension ref="B2:O89"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="9.140625" style="2"/>
@@ -1289,81 +1444,84 @@
     <col min="8" max="8" width="13.28515625" style="2" customWidth="1"/>
     <col min="9" max="10" width="9.140625" style="2"/>
     <col min="11" max="11" width="33.7109375" style="2" customWidth="1"/>
-    <col min="12" max="12" width="27" style="2" customWidth="1"/>
-    <col min="13" max="13" width="11.7109375" style="2" customWidth="1"/>
-    <col min="14" max="14" width="27.7109375" style="2" customWidth="1"/>
-    <col min="15" max="16384" width="9.140625" style="2"/>
+    <col min="12" max="12" width="17.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.7109375" style="2" customWidth="1"/>
+    <col min="15" max="15" width="27.7109375" style="2" customWidth="1"/>
+    <col min="16" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B2" s="12" t="s">
+    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B2" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="H2" s="12" t="s">
+      <c r="H2" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="11" t="s">
         <v>85</v>
       </c>
       <c r="K2" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="L2" s="54" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B3" s="38" t="s">
+      <c r="M2" s="53"/>
+    </row>
+    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B3" s="46" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="45">
+      <c r="C3" s="48">
         <v>1</v>
       </c>
-      <c r="D3" s="42" t="s">
+      <c r="D3" s="40" t="s">
         <v>90</v>
       </c>
-      <c r="E3" s="42" t="s">
+      <c r="E3" s="40" t="s">
         <v>70</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="G3" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="H3" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I3" s="16" t="s">
+      <c r="H3" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="I3" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="K3" s="38" t="s">
+      <c r="K3" s="46" t="s">
         <v>94</v>
       </c>
-      <c r="L3" s="22" t="s">
+      <c r="L3" s="48" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B4" s="38"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="43"/>
+      <c r="M3" s="55"/>
+    </row>
+    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B4" s="46"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
       <c r="F4" s="2" t="s">
         <v>2</v>
       </c>
@@ -1373,19 +1531,20 @@
       <c r="H4" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I4" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="K4" s="38"/>
-      <c r="L4" s="23" t="s">
+      <c r="K4" s="46"/>
+      <c r="L4" s="47" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="38"/>
-      <c r="C5" s="46"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="43"/>
+      <c r="M4" s="56"/>
+    </row>
+    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B5" s="46"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="41"/>
       <c r="F5" s="2" t="s">
         <v>3</v>
       </c>
@@ -1395,21 +1554,22 @@
       <c r="H5" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="K5" s="13" t="s">
+      <c r="K5" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="L5" s="13" t="s">
+      <c r="L5" s="57" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B6" s="38"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="43"/>
-      <c r="E6" s="43"/>
+      <c r="M5" s="58"/>
+    </row>
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B6" s="46"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
       <c r="F6" s="2" t="s">
         <v>64</v>
       </c>
@@ -1419,49 +1579,51 @@
       <c r="H6" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="I6" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="K6" s="38" t="s">
+      <c r="K6" s="46" t="s">
         <v>101</v>
       </c>
-      <c r="L6" s="22" t="s">
+      <c r="L6" s="48" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B7" s="38"/>
-      <c r="C7" s="45">
+      <c r="M6" s="55"/>
+    </row>
+    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B7" s="46"/>
+      <c r="C7" s="48">
         <v>2</v>
       </c>
-      <c r="D7" s="42" t="s">
+      <c r="D7" s="40" t="s">
         <v>91</v>
       </c>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="40" t="s">
         <v>71</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="G7" s="15" t="s">
+      <c r="G7" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="H7" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I7" s="16" t="s">
+      <c r="H7" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="I7" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="K7" s="38"/>
-      <c r="L7" s="23" t="s">
+      <c r="K7" s="46"/>
+      <c r="L7" s="47" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B8" s="38"/>
-      <c r="C8" s="46"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="43"/>
+      <c r="M7" s="56"/>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B8" s="46"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="41"/>
+      <c r="E8" s="41"/>
       <c r="F8" s="2" t="s">
         <v>2</v>
       </c>
@@ -1471,21 +1633,22 @@
       <c r="H8" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="I8" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="K8" s="13" t="s">
+      <c r="K8" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="L8" s="13" t="s">
+      <c r="L8" s="57" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B9" s="38"/>
-      <c r="C9" s="46"/>
-      <c r="D9" s="43"/>
-      <c r="E9" s="43"/>
+      <c r="M8" s="58"/>
+    </row>
+    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B9" s="46"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="41"/>
+      <c r="E9" s="41"/>
       <c r="F9" s="2" t="s">
         <v>3</v>
       </c>
@@ -1495,67 +1658,80 @@
       <c r="H9" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="I9" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="K9" s="13" t="s">
+      <c r="K9" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="L9" s="10" t="s">
+      <c r="L9" s="57" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B10" s="38"/>
+      <c r="M9" s="58"/>
+    </row>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B10" s="46"/>
       <c r="C10" s="47"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="9" t="s">
+      <c r="D10" s="42"/>
+      <c r="E10" s="42"/>
+      <c r="F10" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="H10" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="I10" s="10" t="s">
+      <c r="H10" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="I10" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="K10" s="39" t="s">
+      <c r="K10" s="36" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="38"/>
-      <c r="C11" s="45">
+      <c r="L10" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="M10" s="21" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B11" s="46"/>
+      <c r="C11" s="48">
         <v>3</v>
       </c>
-      <c r="D11" s="42" t="s">
+      <c r="D11" s="40" t="s">
         <v>91</v>
       </c>
-      <c r="E11" s="42" t="s">
+      <c r="E11" s="40" t="s">
         <v>71</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="G11" s="15" t="s">
+      <c r="G11" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="H11" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I11" s="16" t="s">
+      <c r="H11" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="I11" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="K11" s="40"/>
-    </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B12" s="38"/>
-      <c r="C12" s="46"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
+      <c r="K11" s="37"/>
+      <c r="L11" s="35" t="s">
+        <v>187</v>
+      </c>
+      <c r="M11" s="35" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B12" s="46"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
       <c r="F12" s="2" t="s">
         <v>2</v>
       </c>
@@ -1565,16 +1741,22 @@
       <c r="H12" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I12" s="7" t="s">
+      <c r="I12" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="K12" s="40"/>
-    </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B13" s="38"/>
-      <c r="C13" s="46"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="43"/>
+      <c r="K12" s="37"/>
+      <c r="L12" s="35" t="s">
+        <v>188</v>
+      </c>
+      <c r="M12" s="35" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B13" s="46"/>
+      <c r="C13" s="38"/>
+      <c r="D13" s="41"/>
+      <c r="E13" s="41"/>
       <c r="F13" s="2" t="s">
         <v>3</v>
       </c>
@@ -1584,60 +1766,78 @@
       <c r="H13" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I13" s="7" t="s">
+      <c r="I13" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="K13" s="40"/>
-    </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B14" s="38"/>
+      <c r="K13" s="37"/>
+      <c r="L13" s="35" t="s">
+        <v>189</v>
+      </c>
+      <c r="M13" s="35" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B14" s="46"/>
       <c r="C14" s="47"/>
-      <c r="D14" s="44"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="9" t="s">
+      <c r="D14" s="42"/>
+      <c r="E14" s="42"/>
+      <c r="F14" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="H14" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="I14" s="10" t="s">
+      <c r="H14" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="I14" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="K14" s="40"/>
-    </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B15" s="38"/>
-      <c r="C15" s="45">
+      <c r="K14" s="37"/>
+      <c r="L14" s="35" t="s">
+        <v>190</v>
+      </c>
+      <c r="M14" s="35" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="15" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B15" s="46"/>
+      <c r="C15" s="48">
         <v>4</v>
       </c>
-      <c r="D15" s="42" t="s">
+      <c r="D15" s="40" t="s">
         <v>90</v>
       </c>
-      <c r="E15" s="42" t="s">
+      <c r="E15" s="40" t="s">
         <v>70</v>
       </c>
-      <c r="F15" s="15" t="s">
+      <c r="F15" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="G15" s="15" t="s">
+      <c r="G15" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="H15" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I15" s="16" t="s">
+      <c r="H15" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="I15" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="K15" s="40"/>
-    </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B16" s="38"/>
-      <c r="C16" s="46"/>
-      <c r="D16" s="43"/>
-      <c r="E16" s="43"/>
+      <c r="K15" s="37"/>
+      <c r="L15" s="35" t="s">
+        <v>191</v>
+      </c>
+      <c r="M15" s="35" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="16" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B16" s="46"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="41"/>
+      <c r="E16" s="41"/>
       <c r="F16" s="2" t="s">
         <v>2</v>
       </c>
@@ -1647,16 +1847,22 @@
       <c r="H16" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I16" s="7" t="s">
+      <c r="I16" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="K16" s="40"/>
-    </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B17" s="38"/>
-      <c r="C17" s="46"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="43"/>
+      <c r="K16" s="37"/>
+      <c r="L16" s="35" t="s">
+        <v>192</v>
+      </c>
+      <c r="M16" s="35" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B17" s="46"/>
+      <c r="C17" s="38"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="41"/>
       <c r="F17" s="2" t="s">
         <v>3</v>
       </c>
@@ -1666,60 +1872,78 @@
       <c r="H17" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I17" s="7" t="s">
+      <c r="I17" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="K17" s="40"/>
-    </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B18" s="38"/>
+      <c r="K17" s="37"/>
+      <c r="L17" s="35" t="s">
+        <v>181</v>
+      </c>
+      <c r="M17" s="35" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B18" s="46"/>
       <c r="C18" s="47"/>
-      <c r="D18" s="44"/>
-      <c r="E18" s="44"/>
-      <c r="F18" s="9" t="s">
+      <c r="D18" s="42"/>
+      <c r="E18" s="42"/>
+      <c r="F18" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="G18" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="H18" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="I18" s="10" t="s">
+      <c r="H18" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="I18" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="K18" s="40"/>
-    </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B19" s="38"/>
-      <c r="C19" s="45">
+      <c r="K18" s="37"/>
+      <c r="L18" s="35" t="s">
+        <v>182</v>
+      </c>
+      <c r="M18" s="35" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B19" s="46"/>
+      <c r="C19" s="48">
         <v>5</v>
       </c>
-      <c r="D19" s="42" t="s">
+      <c r="D19" s="40" t="s">
         <v>90</v>
       </c>
-      <c r="E19" s="42" t="s">
+      <c r="E19" s="40" t="s">
         <v>70</v>
       </c>
-      <c r="F19" s="15" t="s">
+      <c r="F19" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="G19" s="15" t="s">
+      <c r="G19" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="H19" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I19" s="16" t="s">
+      <c r="H19" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="I19" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="K19" s="40"/>
-    </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B20" s="38"/>
-      <c r="C20" s="46"/>
-      <c r="D20" s="43"/>
-      <c r="E20" s="43"/>
+      <c r="K19" s="37"/>
+      <c r="L19" s="35" t="s">
+        <v>193</v>
+      </c>
+      <c r="M19" s="35" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B20" s="46"/>
+      <c r="C20" s="38"/>
+      <c r="D20" s="41"/>
+      <c r="E20" s="41"/>
       <c r="F20" s="2" t="s">
         <v>2</v>
       </c>
@@ -1729,16 +1953,22 @@
       <c r="H20" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I20" s="7" t="s">
+      <c r="I20" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="K20" s="40"/>
-    </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B21" s="38"/>
-      <c r="C21" s="46"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="43"/>
+      <c r="K20" s="37"/>
+      <c r="L20" s="35" t="s">
+        <v>183</v>
+      </c>
+      <c r="M20" s="35" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B21" s="46"/>
+      <c r="C21" s="38"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
       <c r="F21" s="2" t="s">
         <v>3</v>
       </c>
@@ -1748,62 +1978,70 @@
       <c r="H21" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I21" s="7" t="s">
+      <c r="I21" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="K21" s="40"/>
-    </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B22" s="38"/>
+      <c r="K21" s="37"/>
+      <c r="L21" s="35" t="s">
+        <v>184</v>
+      </c>
+      <c r="M21" s="35" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B22" s="46"/>
       <c r="C22" s="47"/>
-      <c r="D22" s="44"/>
-      <c r="E22" s="44"/>
-      <c r="F22" s="9" t="s">
+      <c r="D22" s="42"/>
+      <c r="E22" s="42"/>
+      <c r="F22" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="G22" s="9" t="s">
+      <c r="G22" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="H22" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="I22" s="10" t="s">
+      <c r="H22" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="I22" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="K22" s="40"/>
-    </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B23" s="38" t="s">
+      <c r="K22" s="37"/>
+      <c r="M22" s="35"/>
+    </row>
+    <row r="23" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B23" s="46" t="s">
         <v>65</v>
       </c>
-      <c r="C23" s="45">
+      <c r="C23" s="48">
         <v>1</v>
       </c>
-      <c r="D23" s="42" t="s">
+      <c r="D23" s="40" t="s">
         <v>90</v>
       </c>
-      <c r="E23" s="42" t="s">
+      <c r="E23" s="40" t="s">
         <v>68</v>
       </c>
-      <c r="F23" s="15" t="s">
+      <c r="F23" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="G23" s="15" t="s">
+      <c r="G23" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="H23" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I23" s="16" t="s">
+      <c r="H23" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="I23" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="K23" s="40"/>
-    </row>
-    <row r="24" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B24" s="38"/>
-      <c r="C24" s="46"/>
-      <c r="D24" s="43"/>
-      <c r="E24" s="43"/>
+      <c r="K23" s="37"/>
+      <c r="M23" s="51"/>
+    </row>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B24" s="46"/>
+      <c r="C24" s="38"/>
+      <c r="D24" s="41"/>
+      <c r="E24" s="41"/>
       <c r="F24" s="2" t="s">
         <v>5</v>
       </c>
@@ -1813,16 +2051,18 @@
       <c r="H24" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I24" s="7" t="s">
+      <c r="I24" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="K24" s="40"/>
-    </row>
-    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B25" s="38"/>
-      <c r="C25" s="46"/>
-      <c r="D25" s="43"/>
-      <c r="E25" s="43"/>
+      <c r="K24" s="37"/>
+      <c r="L24" s="51"/>
+      <c r="M24" s="51"/>
+    </row>
+    <row r="25" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B25" s="46"/>
+      <c r="C25" s="38"/>
+      <c r="D25" s="41"/>
+      <c r="E25" s="41"/>
       <c r="F25" s="2" t="s">
         <v>6</v>
       </c>
@@ -1832,16 +2072,18 @@
       <c r="H25" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I25" s="7" t="s">
+      <c r="I25" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="K25" s="40"/>
-    </row>
-    <row r="26" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B26" s="38"/>
-      <c r="C26" s="46"/>
-      <c r="D26" s="43"/>
-      <c r="E26" s="43"/>
+      <c r="K25" s="37"/>
+      <c r="L25" s="51"/>
+      <c r="M25" s="51"/>
+    </row>
+    <row r="26" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B26" s="46"/>
+      <c r="C26" s="38"/>
+      <c r="D26" s="41"/>
+      <c r="E26" s="41"/>
       <c r="F26" s="2" t="s">
         <v>7</v>
       </c>
@@ -1851,16 +2093,18 @@
       <c r="H26" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I26" s="7" t="s">
+      <c r="I26" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="K26" s="41"/>
-    </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B27" s="38"/>
-      <c r="C27" s="46"/>
-      <c r="D27" s="43"/>
-      <c r="E27" s="43"/>
+      <c r="K26" s="39"/>
+      <c r="L26" s="52"/>
+      <c r="M26" s="52"/>
+    </row>
+    <row r="27" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B27" s="46"/>
+      <c r="C27" s="38"/>
+      <c r="D27" s="41"/>
+      <c r="E27" s="41"/>
       <c r="F27" s="2" t="s">
         <v>8</v>
       </c>
@@ -1870,42 +2114,43 @@
       <c r="H27" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I27" s="7" t="s">
+      <c r="I27" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="K27" s="13" t="s">
+      <c r="K27" s="12" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="28" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B28" s="38"/>
-      <c r="C28" s="45">
+      <c r="L27" s="50"/>
+    </row>
+    <row r="28" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B28" s="46"/>
+      <c r="C28" s="48">
         <v>2</v>
       </c>
-      <c r="D28" s="42" t="s">
+      <c r="D28" s="40" t="s">
         <v>91</v>
       </c>
-      <c r="E28" s="42" t="s">
+      <c r="E28" s="40" t="s">
         <v>69</v>
       </c>
-      <c r="F28" s="15" t="s">
+      <c r="F28" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="G28" s="15" t="s">
+      <c r="G28" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="H28" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I28" s="16" t="s">
+      <c r="H28" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="I28" s="15" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="29" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B29" s="38"/>
-      <c r="C29" s="46"/>
-      <c r="D29" s="43"/>
-      <c r="E29" s="43"/>
+    <row r="29" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B29" s="46"/>
+      <c r="C29" s="38"/>
+      <c r="D29" s="41"/>
+      <c r="E29" s="41"/>
       <c r="F29" s="2" t="s">
         <v>5</v>
       </c>
@@ -1915,15 +2160,15 @@
       <c r="H29" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I29" s="7" t="s">
+      <c r="I29" s="6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B30" s="38"/>
-      <c r="C30" s="46"/>
-      <c r="D30" s="43"/>
-      <c r="E30" s="43"/>
+    <row r="30" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B30" s="46"/>
+      <c r="C30" s="38"/>
+      <c r="D30" s="41"/>
+      <c r="E30" s="41"/>
       <c r="F30" s="2" t="s">
         <v>6</v>
       </c>
@@ -1933,15 +2178,15 @@
       <c r="H30" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I30" s="7" t="s">
+      <c r="I30" s="6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B31" s="38"/>
-      <c r="C31" s="46"/>
-      <c r="D31" s="43"/>
-      <c r="E31" s="43"/>
+    <row r="31" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B31" s="46"/>
+      <c r="C31" s="38"/>
+      <c r="D31" s="41"/>
+      <c r="E31" s="41"/>
       <c r="F31" s="2" t="s">
         <v>7</v>
       </c>
@@ -1951,65 +2196,66 @@
       <c r="H31" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I31" s="7" t="s">
+      <c r="I31" s="6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="32" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B32" s="38"/>
+    <row r="32" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B32" s="46"/>
       <c r="C32" s="47"/>
-      <c r="D32" s="44"/>
-      <c r="E32" s="44"/>
-      <c r="F32" s="9" t="s">
+      <c r="D32" s="42"/>
+      <c r="E32" s="42"/>
+      <c r="F32" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="G32" s="9" t="s">
+      <c r="G32" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="H32" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="I32" s="10" t="s">
+      <c r="H32" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="I32" s="9" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="33" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B33" s="38"/>
-      <c r="C33" s="45">
+    <row r="33" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B33" s="46"/>
+      <c r="C33" s="48">
         <v>3</v>
       </c>
-      <c r="D33" s="42" t="s">
+      <c r="D33" s="40" t="s">
         <v>91</v>
       </c>
-      <c r="E33" s="42" t="s">
+      <c r="E33" s="40" t="s">
         <v>69</v>
       </c>
-      <c r="F33" s="15" t="s">
+      <c r="F33" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="G33" s="15" t="s">
+      <c r="G33" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="H33" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I33" s="16" t="s">
+      <c r="H33" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="I33" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="K33" s="37" t="s">
+      <c r="K33" s="49" t="s">
         <v>112</v>
       </c>
-      <c r="L33" s="37"/>
-      <c r="M33" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="N33" s="1"/>
-    </row>
-    <row r="34" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B34" s="38"/>
-      <c r="C34" s="46"/>
-      <c r="D34" s="43"/>
-      <c r="E34" s="43"/>
+      <c r="L33" s="49"/>
+      <c r="M33" s="49"/>
+      <c r="N33" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="O33" s="1"/>
+    </row>
+    <row r="34" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B34" s="46"/>
+      <c r="C34" s="38"/>
+      <c r="D34" s="41"/>
+      <c r="E34" s="41"/>
       <c r="F34" s="2" t="s">
         <v>5</v>
       </c>
@@ -2019,24 +2265,25 @@
       <c r="H34" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I34" s="7" t="s">
+      <c r="I34" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="K34" s="36" t="s">
-        <v>150</v>
-      </c>
-      <c r="L34" s="36" t="s">
-        <v>158</v>
-      </c>
-      <c r="M34" s="36" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="35" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B35" s="38"/>
-      <c r="C35" s="46"/>
-      <c r="D35" s="43"/>
-      <c r="E35" s="43"/>
+      <c r="K34" s="34" t="s">
+        <v>149</v>
+      </c>
+      <c r="L34" s="59" t="s">
+        <v>167</v>
+      </c>
+      <c r="M34" s="59"/>
+      <c r="N34" s="34" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="35" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B35" s="46"/>
+      <c r="C35" s="38"/>
+      <c r="D35" s="41"/>
+      <c r="E35" s="41"/>
       <c r="F35" s="2" t="s">
         <v>6</v>
       </c>
@@ -2046,24 +2293,25 @@
       <c r="H35" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I35" s="7" t="s">
+      <c r="I35" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="K35" s="36" t="s">
-        <v>152</v>
-      </c>
-      <c r="L35" s="36" t="s">
-        <v>168</v>
-      </c>
-      <c r="M35" s="36" t="s">
+      <c r="K35" s="34" t="s">
+        <v>151</v>
+      </c>
+      <c r="L35" s="59" t="s">
+        <v>201</v>
+      </c>
+      <c r="M35" s="59"/>
+      <c r="N35" s="34" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="36" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B36" s="38"/>
-      <c r="C36" s="46"/>
-      <c r="D36" s="43"/>
-      <c r="E36" s="43"/>
+    <row r="36" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B36" s="46"/>
+      <c r="C36" s="38"/>
+      <c r="D36" s="41"/>
+      <c r="E36" s="41"/>
       <c r="F36" s="2" t="s">
         <v>7</v>
       </c>
@@ -2073,84 +2321,87 @@
       <c r="H36" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I36" s="7" t="s">
+      <c r="I36" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="K36" s="36" t="s">
-        <v>157</v>
-      </c>
-      <c r="L36" s="36" t="s">
-        <v>160</v>
-      </c>
-      <c r="M36" s="36" t="s">
+      <c r="K36" s="34" t="s">
+        <v>156</v>
+      </c>
+      <c r="L36" s="59" t="s">
+        <v>159</v>
+      </c>
+      <c r="M36" s="59"/>
+      <c r="N36" s="34" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="37" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B37" s="46"/>
+      <c r="C37" s="47"/>
+      <c r="D37" s="42"/>
+      <c r="E37" s="42"/>
+      <c r="F37" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="G37" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="H37" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="I37" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="K37" s="34" t="s">
+        <v>113</v>
+      </c>
+      <c r="L37" s="59" t="s">
+        <v>158</v>
+      </c>
+      <c r="M37" s="59"/>
+      <c r="N37" s="34" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="38" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B38" s="46"/>
+      <c r="C38" s="48">
+        <v>6</v>
+      </c>
+      <c r="D38" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="E38" s="40" t="s">
+        <v>68</v>
+      </c>
+      <c r="F38" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="G38" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="H38" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="I38" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="K38" s="34" t="s">
+        <v>171</v>
+      </c>
+      <c r="L38" s="59" t="s">
+        <v>155</v>
+      </c>
+      <c r="M38" s="59"/>
+      <c r="N38" s="34" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="37" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B37" s="38"/>
-      <c r="C37" s="47"/>
-      <c r="D37" s="44"/>
-      <c r="E37" s="44"/>
-      <c r="F37" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="G37" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="H37" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="I37" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="K37" s="36" t="s">
-        <v>114</v>
-      </c>
-      <c r="L37" s="36" t="s">
-        <v>159</v>
-      </c>
-      <c r="M37" s="36" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="38" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B38" s="38"/>
-      <c r="C38" s="45">
-        <v>6</v>
-      </c>
-      <c r="D38" s="42" t="s">
-        <v>90</v>
-      </c>
-      <c r="E38" s="42" t="s">
-        <v>68</v>
-      </c>
-      <c r="F38" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="G38" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="H38" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I38" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="K38" s="36" t="s">
-        <v>113</v>
-      </c>
-      <c r="L38" s="36" t="s">
-        <v>156</v>
-      </c>
-      <c r="M38" s="36" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="39" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B39" s="38"/>
-      <c r="C39" s="46"/>
-      <c r="D39" s="43"/>
-      <c r="E39" s="43"/>
+    <row r="39" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B39" s="46"/>
+      <c r="C39" s="38"/>
+      <c r="D39" s="41"/>
+      <c r="E39" s="41"/>
       <c r="F39" s="2" t="s">
         <v>5</v>
       </c>
@@ -2160,24 +2411,25 @@
       <c r="H39" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I39" s="7" t="s">
+      <c r="I39" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="K39" s="36" t="s">
-        <v>115</v>
-      </c>
-      <c r="L39" s="36" t="s">
-        <v>154</v>
-      </c>
-      <c r="M39" s="36" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="40" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B40" s="38"/>
-      <c r="C40" s="46"/>
-      <c r="D40" s="43"/>
-      <c r="E40" s="43"/>
+      <c r="K39" s="34" t="s">
+        <v>114</v>
+      </c>
+      <c r="L39" s="59" t="s">
+        <v>157</v>
+      </c>
+      <c r="M39" s="59"/>
+      <c r="N39" s="34" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="40" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B40" s="46"/>
+      <c r="C40" s="38"/>
+      <c r="D40" s="41"/>
+      <c r="E40" s="41"/>
       <c r="F40" s="2" t="s">
         <v>6</v>
       </c>
@@ -2187,24 +2439,25 @@
       <c r="H40" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I40" s="7" t="s">
+      <c r="I40" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="K40" s="36" t="s">
-        <v>151</v>
-      </c>
-      <c r="L40" s="36" t="s">
-        <v>169</v>
-      </c>
-      <c r="M40" s="36" t="s">
+      <c r="K40" s="34" t="s">
+        <v>150</v>
+      </c>
+      <c r="L40" s="59" t="s">
+        <v>168</v>
+      </c>
+      <c r="M40" s="59"/>
+      <c r="N40" s="34" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="41" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B41" s="38"/>
-      <c r="C41" s="46"/>
-      <c r="D41" s="43"/>
-      <c r="E41" s="43"/>
+    <row r="41" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B41" s="46"/>
+      <c r="C41" s="38"/>
+      <c r="D41" s="41"/>
+      <c r="E41" s="41"/>
       <c r="F41" s="2" t="s">
         <v>7</v>
       </c>
@@ -2214,77 +2467,89 @@
       <c r="H41" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I41" s="7" t="s">
+      <c r="I41" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="K41" s="36" t="s">
-        <v>155</v>
-      </c>
-      <c r="L41" s="36" t="s">
-        <v>162</v>
-      </c>
-      <c r="M41" s="36" t="s">
+      <c r="K41" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="L41" s="59" t="s">
+        <v>161</v>
+      </c>
+      <c r="M41" s="59"/>
+      <c r="N41" s="34" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="42" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B42" s="38"/>
+    <row r="42" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B42" s="46"/>
       <c r="C42" s="47"/>
-      <c r="D42" s="44"/>
-      <c r="E42" s="44"/>
-      <c r="F42" s="9" t="s">
+      <c r="D42" s="42"/>
+      <c r="E42" s="42"/>
+      <c r="F42" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="G42" s="9" t="s">
+      <c r="G42" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="H42" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="I42" s="10" t="s">
+      <c r="H42" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="I42" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="K42" s="36" t="s">
-        <v>153</v>
-      </c>
-      <c r="L42" s="36" t="s">
-        <v>161</v>
-      </c>
-      <c r="M42" s="36" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="43" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B43" s="38" t="s">
+      <c r="K42" s="34" t="s">
+        <v>152</v>
+      </c>
+      <c r="L42" s="59" t="s">
+        <v>160</v>
+      </c>
+      <c r="M42" s="59"/>
+      <c r="N42" s="34" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="43" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B43" s="46" t="s">
         <v>66</v>
       </c>
-      <c r="C43" s="45">
+      <c r="C43" s="48">
         <v>1</v>
       </c>
-      <c r="D43" s="42" t="s">
+      <c r="D43" s="40" t="s">
         <v>91</v>
       </c>
-      <c r="E43" s="48" t="s">
+      <c r="E43" s="43" t="s">
         <v>92</v>
       </c>
-      <c r="F43" s="15" t="s">
+      <c r="F43" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="G43" s="15" t="s">
+      <c r="G43" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="H43" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I43" s="16" t="s">
+      <c r="H43" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="I43" s="15" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="44" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B44" s="38"/>
-      <c r="C44" s="46"/>
-      <c r="D44" s="43"/>
-      <c r="E44" s="49"/>
+      <c r="K43" s="22" t="s">
+        <v>169</v>
+      </c>
+      <c r="L43" s="59" t="s">
+        <v>204</v>
+      </c>
+      <c r="M43" s="59"/>
+      <c r="N43" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="44" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B44" s="46"/>
+      <c r="C44" s="38"/>
+      <c r="D44" s="41"/>
+      <c r="E44" s="44"/>
       <c r="F44" s="2" t="s">
         <v>10</v>
       </c>
@@ -2294,57 +2559,87 @@
       <c r="H44" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I44" s="7" t="s">
+      <c r="I44" s="6" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="45" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B45" s="38"/>
+      <c r="K44" s="34" t="s">
+        <v>172</v>
+      </c>
+      <c r="L44" s="59" t="s">
+        <v>205</v>
+      </c>
+      <c r="M44" s="59"/>
+      <c r="N44" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="45" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B45" s="46"/>
       <c r="C45" s="47"/>
-      <c r="D45" s="44"/>
-      <c r="E45" s="50"/>
-      <c r="F45" s="9" t="s">
+      <c r="D45" s="42"/>
+      <c r="E45" s="45"/>
+      <c r="F45" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G45" s="9" t="s">
+      <c r="G45" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="H45" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="I45" s="10" t="s">
+      <c r="H45" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="I45" s="9" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="46" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B46" s="38"/>
-      <c r="C46" s="45">
+      <c r="K45" s="34" t="s">
+        <v>173</v>
+      </c>
+      <c r="L45" s="59" t="s">
+        <v>206</v>
+      </c>
+      <c r="M45" s="59"/>
+      <c r="N45" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="46" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B46" s="46"/>
+      <c r="C46" s="48">
         <v>2</v>
       </c>
-      <c r="D46" s="42" t="s">
+      <c r="D46" s="40" t="s">
         <v>91</v>
       </c>
-      <c r="E46" s="42" t="s">
+      <c r="E46" s="40" t="s">
         <v>67</v>
       </c>
-      <c r="F46" s="15" t="s">
+      <c r="F46" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="G46" s="15" t="s">
+      <c r="G46" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="H46" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I46" s="16" t="s">
+      <c r="H46" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="I46" s="15" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="47" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B47" s="38"/>
-      <c r="C47" s="46"/>
-      <c r="D47" s="43"/>
-      <c r="E47" s="43"/>
+      <c r="K46" s="34" t="s">
+        <v>174</v>
+      </c>
+      <c r="L46" s="59" t="s">
+        <v>207</v>
+      </c>
+      <c r="M46" s="59"/>
+      <c r="N46" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="47" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B47" s="46"/>
+      <c r="C47" s="38"/>
+      <c r="D47" s="41"/>
+      <c r="E47" s="41"/>
       <c r="F47" s="2" t="s">
         <v>10</v>
       </c>
@@ -2354,37 +2649,57 @@
       <c r="H47" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I47" s="7" t="s">
+      <c r="I47" s="6" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="48" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B48" s="38"/>
+      <c r="K47" s="34" t="s">
+        <v>175</v>
+      </c>
+      <c r="L47" s="59" t="s">
+        <v>208</v>
+      </c>
+      <c r="M47" s="59"/>
+      <c r="N47" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="48" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B48" s="46"/>
       <c r="C48" s="47"/>
-      <c r="D48" s="44"/>
-      <c r="E48" s="44"/>
-      <c r="F48" s="9" t="s">
+      <c r="D48" s="42"/>
+      <c r="E48" s="42"/>
+      <c r="F48" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G48" s="9" t="s">
+      <c r="G48" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="H48" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="I48" s="10" t="s">
+      <c r="H48" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="I48" s="9" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="49" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B49" s="38"/>
-      <c r="C49" s="46">
+      <c r="K48" s="34" t="s">
+        <v>180</v>
+      </c>
+      <c r="L48" s="59" t="s">
+        <v>209</v>
+      </c>
+      <c r="M48" s="59"/>
+      <c r="N48" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="49" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B49" s="46"/>
+      <c r="C49" s="38">
         <v>3</v>
       </c>
-      <c r="D49" s="43" t="s">
+      <c r="D49" s="41" t="s">
         <v>91</v>
       </c>
-      <c r="E49" s="43" t="s">
+      <c r="E49" s="41" t="s">
         <v>67</v>
       </c>
       <c r="F49" s="2" t="s">
@@ -2396,15 +2711,25 @@
       <c r="H49" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I49" s="7" t="s">
+      <c r="I49" s="6" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="50" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B50" s="38"/>
-      <c r="C50" s="46"/>
-      <c r="D50" s="43"/>
-      <c r="E50" s="43"/>
+      <c r="K49" s="34" t="s">
+        <v>176</v>
+      </c>
+      <c r="L49" s="59" t="s">
+        <v>210</v>
+      </c>
+      <c r="M49" s="59"/>
+      <c r="N49" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="50" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B50" s="46"/>
+      <c r="C50" s="38"/>
+      <c r="D50" s="41"/>
+      <c r="E50" s="41"/>
       <c r="F50" s="2" t="s">
         <v>10</v>
       </c>
@@ -2414,59 +2739,89 @@
       <c r="H50" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I50" s="7" t="s">
+      <c r="I50" s="6" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="51" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B51" s="38"/>
+      <c r="K50" s="34" t="s">
+        <v>177</v>
+      </c>
+      <c r="L50" s="59" t="s">
+        <v>211</v>
+      </c>
+      <c r="M50" s="59"/>
+      <c r="N50" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="51" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B51" s="46"/>
       <c r="C51" s="47"/>
-      <c r="D51" s="44"/>
-      <c r="E51" s="44"/>
-      <c r="F51" s="9" t="s">
+      <c r="D51" s="42"/>
+      <c r="E51" s="42"/>
+      <c r="F51" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G51" s="9" t="s">
+      <c r="G51" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="H51" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="I51" s="10" t="s">
+      <c r="H51" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="I51" s="9" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="52" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B52" s="38" t="s">
+      <c r="K51" s="34" t="s">
+        <v>178</v>
+      </c>
+      <c r="L51" s="59" t="s">
+        <v>212</v>
+      </c>
+      <c r="M51" s="59"/>
+      <c r="N51" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="52" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B52" s="46" t="s">
         <v>83</v>
       </c>
-      <c r="C52" s="18">
+      <c r="C52" s="17">
         <v>0</v>
       </c>
-      <c r="D52" s="15" t="s">
+      <c r="D52" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="E52" s="15" t="str">
+      <c r="E52" s="14" t="str">
         <f>"-"</f>
         <v>-</v>
       </c>
-      <c r="F52" s="17" t="s">
+      <c r="F52" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="G52" s="17" t="s">
+      <c r="G52" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="H52" s="15" t="s">
+      <c r="H52" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="I52" s="16" t="str">
+      <c r="I52" s="15" t="str">
         <f>"-"</f>
         <v>-</v>
       </c>
-    </row>
-    <row r="53" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B53" s="38"/>
-      <c r="C53" s="19">
+      <c r="K52" s="34" t="s">
+        <v>179</v>
+      </c>
+      <c r="L52" s="59" t="s">
+        <v>213</v>
+      </c>
+      <c r="M52" s="59"/>
+      <c r="N52" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="53" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B53" s="46"/>
+      <c r="C53" s="18">
         <v>1</v>
       </c>
       <c r="D53" s="2" t="s">
@@ -2476,23 +2831,29 @@
         <f t="shared" ref="E53:E67" si="0">"-"</f>
         <v>-</v>
       </c>
-      <c r="F53" s="8" t="s">
+      <c r="F53" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G53" s="8" t="s">
+      <c r="G53" s="7" t="s">
         <v>73</v>
       </c>
       <c r="H53" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I53" s="7" t="str">
+      <c r="I53" s="6" t="str">
         <f t="shared" ref="I53:I67" si="1">"-"</f>
         <v>-</v>
       </c>
-    </row>
-    <row r="54" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B54" s="38"/>
-      <c r="C54" s="19">
+      <c r="K53" s="49" t="s">
+        <v>202</v>
+      </c>
+      <c r="L53" s="49"/>
+      <c r="M53" s="49"/>
+      <c r="N53" s="49"/>
+    </row>
+    <row r="54" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B54" s="46"/>
+      <c r="C54" s="18">
         <v>2</v>
       </c>
       <c r="D54" s="2" t="s">
@@ -2502,23 +2863,26 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="F54" s="8" t="s">
+      <c r="F54" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G54" s="8" t="s">
+      <c r="G54" s="7" t="s">
         <v>74</v>
       </c>
       <c r="H54" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I54" s="7" t="str">
+      <c r="I54" s="6" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="55" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B55" s="38"/>
-      <c r="C55" s="19">
+      <c r="K54" s="34" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="55" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B55" s="46"/>
+      <c r="C55" s="18">
         <v>3</v>
       </c>
       <c r="D55" s="2" t="s">
@@ -2528,23 +2892,26 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="F55" s="8" t="s">
+      <c r="F55" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G55" s="8" t="s">
+      <c r="G55" s="7" t="s">
         <v>75</v>
       </c>
       <c r="H55" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I55" s="7" t="str">
+      <c r="I55" s="6" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
-    </row>
-    <row r="56" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B56" s="38"/>
-      <c r="C56" s="19">
+      <c r="K55" s="34" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="56" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B56" s="46"/>
+      <c r="C56" s="18">
         <v>4</v>
       </c>
       <c r="D56" s="2" t="s">
@@ -2554,23 +2921,23 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="F56" s="8" t="s">
+      <c r="F56" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G56" s="8" t="s">
+      <c r="G56" s="7" t="s">
         <v>15</v>
       </c>
       <c r="H56" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I56" s="7" t="str">
+      <c r="I56" s="6" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="57" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B57" s="38"/>
-      <c r="C57" s="19">
+    <row r="57" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B57" s="46"/>
+      <c r="C57" s="18">
         <v>5</v>
       </c>
       <c r="D57" s="2" t="s">
@@ -2580,23 +2947,23 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="F57" s="8" t="s">
+      <c r="F57" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G57" s="8" t="s">
+      <c r="G57" s="7" t="s">
         <v>12</v>
       </c>
       <c r="H57" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I57" s="7" t="str">
+      <c r="I57" s="6" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="58" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B58" s="38"/>
-      <c r="C58" s="19">
+    <row r="58" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B58" s="46"/>
+      <c r="C58" s="18">
         <v>6</v>
       </c>
       <c r="D58" s="2" t="s">
@@ -2606,23 +2973,23 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="F58" s="8" t="s">
+      <c r="F58" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G58" s="8" t="s">
+      <c r="G58" s="7" t="s">
         <v>13</v>
       </c>
       <c r="H58" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I58" s="7" t="str">
+      <c r="I58" s="6" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="59" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B59" s="38"/>
-      <c r="C59" s="19">
+    <row r="59" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B59" s="46"/>
+      <c r="C59" s="18">
         <v>7</v>
       </c>
       <c r="D59" s="2" t="s">
@@ -2632,23 +2999,23 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="F59" s="8" t="s">
+      <c r="F59" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G59" s="8" t="s">
+      <c r="G59" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H59" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I59" s="7" t="str">
+      <c r="I59" s="6" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="60" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B60" s="38"/>
-      <c r="C60" s="19">
+    <row r="60" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B60" s="46"/>
+      <c r="C60" s="18">
         <v>8</v>
       </c>
       <c r="D60" s="2" t="s">
@@ -2658,23 +3025,23 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="F60" s="8" t="s">
+      <c r="F60" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G60" s="8" t="s">
+      <c r="G60" s="7" t="s">
         <v>28</v>
       </c>
       <c r="H60" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I60" s="7" t="str">
+      <c r="I60" s="6" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="61" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B61" s="38"/>
-      <c r="C61" s="19">
+    <row r="61" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B61" s="46"/>
+      <c r="C61" s="18">
         <v>9</v>
       </c>
       <c r="D61" s="2" t="s">
@@ -2684,23 +3051,23 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="F61" s="8" t="s">
+      <c r="F61" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G61" s="8" t="s">
+      <c r="G61" s="7" t="s">
         <v>76</v>
       </c>
       <c r="H61" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I61" s="7" t="str">
+      <c r="I61" s="6" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="62" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B62" s="38"/>
-      <c r="C62" s="19">
+    <row r="62" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B62" s="46"/>
+      <c r="C62" s="18">
         <v>10</v>
       </c>
       <c r="D62" s="2" t="s">
@@ -2710,23 +3077,23 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="F62" s="8" t="s">
+      <c r="F62" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G62" s="8" t="s">
+      <c r="G62" s="7" t="s">
         <v>77</v>
       </c>
       <c r="H62" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I62" s="7" t="str">
+      <c r="I62" s="6" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="63" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B63" s="38"/>
-      <c r="C63" s="19">
+    <row r="63" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B63" s="46"/>
+      <c r="C63" s="18">
         <v>11</v>
       </c>
       <c r="D63" s="2" t="s">
@@ -2736,26 +3103,27 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="F63" s="8" t="s">
+      <c r="F63" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G63" s="8" t="s">
+      <c r="G63" s="7" t="s">
         <v>78</v>
       </c>
       <c r="H63" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I63" s="7" t="str">
+      <c r="I63" s="6" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="K63" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="64" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B64" s="38"/>
-      <c r="C64" s="19">
+      <c r="L63" s="3"/>
+    </row>
+    <row r="64" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B64" s="46"/>
+      <c r="C64" s="18">
         <v>12</v>
       </c>
       <c r="D64" s="2" t="s">
@@ -2765,26 +3133,27 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="F64" s="8" t="s">
+      <c r="F64" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G64" s="8" t="s">
+      <c r="G64" s="7" t="s">
         <v>79</v>
       </c>
       <c r="H64" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I64" s="7" t="str">
+      <c r="I64" s="6" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="K64" s="3" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="65" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B65" s="38"/>
-      <c r="C65" s="19">
+      <c r="L64" s="3"/>
+    </row>
+    <row r="65" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B65" s="46"/>
+      <c r="C65" s="18">
         <v>13</v>
       </c>
       <c r="D65" s="2" t="s">
@@ -2794,23 +3163,23 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="F65" s="8" t="s">
+      <c r="F65" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G65" s="8" t="s">
+      <c r="G65" s="7" t="s">
         <v>80</v>
       </c>
       <c r="H65" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I65" s="7" t="str">
+      <c r="I65" s="6" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="66" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B66" s="38"/>
-      <c r="C66" s="19">
+    <row r="66" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B66" s="46"/>
+      <c r="C66" s="18">
         <v>14</v>
       </c>
       <c r="D66" s="2" t="s">
@@ -2820,82 +3189,84 @@
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="F66" s="8" t="s">
+      <c r="F66" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G66" s="8" t="s">
+      <c r="G66" s="7" t="s">
         <v>81</v>
       </c>
       <c r="H66" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I66" s="7" t="str">
+      <c r="I66" s="6" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
     </row>
-    <row r="67" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B67" s="38"/>
-      <c r="C67" s="20">
+    <row r="67" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B67" s="46"/>
+      <c r="C67" s="19">
         <v>15</v>
       </c>
-      <c r="D67" s="9" t="s">
+      <c r="D67" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="E67" s="9" t="str">
+      <c r="E67" s="8" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
-      <c r="F67" s="21" t="s">
+      <c r="F67" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="G67" s="21" t="s">
+      <c r="G67" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="H67" s="9" t="s">
+      <c r="H67" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="I67" s="10" t="str">
+      <c r="I67" s="9" t="str">
         <f t="shared" si="1"/>
         <v>-</v>
       </c>
       <c r="J67"/>
       <c r="K67"/>
-    </row>
-    <row r="68" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B68" s="39" t="s">
+      <c r="L67"/>
+    </row>
+    <row r="68" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B68" s="36" t="s">
         <v>94</v>
       </c>
-      <c r="C68" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="D68" s="15" t="str">
+      <c r="C68" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="D68" s="14" t="str">
         <f t="shared" ref="D68:E81" si="2">"-"</f>
         <v>-</v>
       </c>
-      <c r="E68" s="15" t="str">
+      <c r="E68" s="14" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="F68" s="15" t="s">
-        <v>116</v>
-      </c>
-      <c r="G68" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="H68" s="15" t="s">
-        <v>87</v>
-      </c>
-      <c r="I68" s="16" t="s">
-        <v>140</v>
+      <c r="F68" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="G68" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="H68" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="I68" s="15" t="s">
+        <v>139</v>
       </c>
       <c r="J68"/>
       <c r="K68"/>
-    </row>
-    <row r="69" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B69" s="40"/>
-      <c r="C69" s="6" t="s">
-        <v>124</v>
+      <c r="L68"/>
+    </row>
+    <row r="69" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B69" s="37"/>
+      <c r="C69" s="5" t="s">
+        <v>123</v>
       </c>
       <c r="D69" s="2" t="str">
         <f t="shared" si="2"/>
@@ -2906,24 +3277,25 @@
         <v>-</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="H69" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I69" s="7" t="s">
-        <v>140</v>
+      <c r="I69" s="6" t="s">
+        <v>139</v>
       </c>
       <c r="J69"/>
       <c r="K69"/>
-    </row>
-    <row r="70" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B70" s="40"/>
-      <c r="C70" s="6" t="s">
-        <v>125</v>
+      <c r="L69"/>
+    </row>
+    <row r="70" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B70" s="37"/>
+      <c r="C70" s="5" t="s">
+        <v>124</v>
       </c>
       <c r="D70" s="2" t="str">
         <f t="shared" si="2"/>
@@ -2934,24 +3306,25 @@
         <v>-</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H70" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I70" s="7" t="s">
-        <v>140</v>
+      <c r="I70" s="6" t="s">
+        <v>139</v>
       </c>
       <c r="J70"/>
       <c r="K70"/>
-    </row>
-    <row r="71" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B71" s="40"/>
-      <c r="C71" s="6" t="s">
-        <v>126</v>
+      <c r="L70"/>
+    </row>
+    <row r="71" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B71" s="37"/>
+      <c r="C71" s="5" t="s">
+        <v>125</v>
       </c>
       <c r="D71" s="2" t="str">
         <f t="shared" si="2"/>
@@ -2962,24 +3335,25 @@
         <v>-</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H71" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I71" s="7" t="s">
-        <v>140</v>
+      <c r="I71" s="6" t="s">
+        <v>139</v>
       </c>
       <c r="J71"/>
       <c r="K71"/>
-    </row>
-    <row r="72" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B72" s="40"/>
-      <c r="C72" s="6" t="s">
-        <v>127</v>
+      <c r="L71"/>
+    </row>
+    <row r="72" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B72" s="37"/>
+      <c r="C72" s="5" t="s">
+        <v>126</v>
       </c>
       <c r="D72" s="2" t="str">
         <f t="shared" si="2"/>
@@ -2990,24 +3364,25 @@
         <v>-</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H72" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I72" s="7" t="s">
-        <v>140</v>
+      <c r="I72" s="6" t="s">
+        <v>139</v>
       </c>
       <c r="J72"/>
       <c r="K72"/>
-    </row>
-    <row r="73" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B73" s="40"/>
-      <c r="C73" s="6" t="s">
-        <v>128</v>
+      <c r="L72"/>
+    </row>
+    <row r="73" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B73" s="37"/>
+      <c r="C73" s="5" t="s">
+        <v>127</v>
       </c>
       <c r="D73" s="2" t="str">
         <f t="shared" si="2"/>
@@ -3018,24 +3393,25 @@
         <v>-</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H73" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I73" s="7" t="s">
-        <v>140</v>
+      <c r="I73" s="6" t="s">
+        <v>139</v>
       </c>
       <c r="J73"/>
       <c r="K73"/>
-    </row>
-    <row r="74" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B74" s="40"/>
-      <c r="C74" s="6" t="s">
-        <v>129</v>
+      <c r="L73"/>
+    </row>
+    <row r="74" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B74" s="37"/>
+      <c r="C74" s="5" t="s">
+        <v>128</v>
       </c>
       <c r="D74" s="2" t="str">
         <f t="shared" si="2"/>
@@ -3046,24 +3422,25 @@
         <v>-</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H74" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I74" s="7" t="s">
-        <v>140</v>
+      <c r="I74" s="6" t="s">
+        <v>139</v>
       </c>
       <c r="J74"/>
       <c r="K74"/>
-    </row>
-    <row r="75" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B75" s="40"/>
-      <c r="C75" s="6" t="s">
-        <v>130</v>
+      <c r="L74"/>
+    </row>
+    <row r="75" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B75" s="37"/>
+      <c r="C75" s="5" t="s">
+        <v>129</v>
       </c>
       <c r="D75" s="2" t="str">
         <f t="shared" si="2"/>
@@ -3074,24 +3451,25 @@
         <v>-</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H75" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I75" s="7" t="s">
-        <v>140</v>
+      <c r="I75" s="6" t="s">
+        <v>139</v>
       </c>
       <c r="J75"/>
       <c r="K75"/>
-    </row>
-    <row r="76" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B76" s="40"/>
-      <c r="C76" s="26" t="s">
-        <v>149</v>
+      <c r="L75"/>
+    </row>
+    <row r="76" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B76" s="37"/>
+      <c r="C76" s="24" t="s">
+        <v>148</v>
       </c>
       <c r="D76" s="2" t="str">
         <f t="shared" si="2"/>
@@ -3102,7 +3480,7 @@
         <v>-</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G76" s="2" t="s">
         <v>41</v>
@@ -3110,16 +3488,17 @@
       <c r="H76" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I76" s="7" t="s">
-        <v>140</v>
+      <c r="I76" s="6" t="s">
+        <v>139</v>
       </c>
       <c r="J76"/>
       <c r="K76"/>
-    </row>
-    <row r="77" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B77" s="40"/>
-      <c r="C77" s="26" t="s">
-        <v>149</v>
+      <c r="L76"/>
+    </row>
+    <row r="77" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B77" s="37"/>
+      <c r="C77" s="24" t="s">
+        <v>148</v>
       </c>
       <c r="D77" s="2" t="str">
         <f t="shared" si="2"/>
@@ -3129,8 +3508,8 @@
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="F77" s="8" t="s">
-        <v>118</v>
+      <c r="F77" s="7" t="s">
+        <v>117</v>
       </c>
       <c r="G77" s="2" t="s">
         <v>42</v>
@@ -3138,16 +3517,17 @@
       <c r="H77" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I77" s="7" t="s">
-        <v>140</v>
+      <c r="I77" s="6" t="s">
+        <v>139</v>
       </c>
       <c r="J77"/>
       <c r="K77"/>
-    </row>
-    <row r="78" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B78" s="40"/>
-      <c r="C78" s="6" t="s">
-        <v>142</v>
+      <c r="L77"/>
+    </row>
+    <row r="78" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B78" s="37"/>
+      <c r="C78" s="5" t="s">
+        <v>141</v>
       </c>
       <c r="D78" s="2" t="str">
         <f t="shared" si="2"/>
@@ -3157,8 +3537,8 @@
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="F78" s="8" t="s">
-        <v>119</v>
+      <c r="F78" s="7" t="s">
+        <v>118</v>
       </c>
       <c r="G78" s="2" t="s">
         <v>34</v>
@@ -3166,16 +3546,17 @@
       <c r="H78" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I78" s="7" t="s">
-        <v>140</v>
+      <c r="I78" s="6" t="s">
+        <v>139</v>
       </c>
       <c r="J78"/>
       <c r="K78"/>
-    </row>
-    <row r="79" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B79" s="40"/>
-      <c r="C79" s="6" t="s">
-        <v>143</v>
+      <c r="L78"/>
+    </row>
+    <row r="79" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B79" s="37"/>
+      <c r="C79" s="5" t="s">
+        <v>142</v>
       </c>
       <c r="D79" s="2" t="str">
         <f t="shared" si="2"/>
@@ -3185,8 +3566,8 @@
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="F79" s="8" t="s">
-        <v>120</v>
+      <c r="F79" s="7" t="s">
+        <v>119</v>
       </c>
       <c r="G79" s="2" t="s">
         <v>37</v>
@@ -3194,44 +3575,46 @@
       <c r="H79" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I79" s="7" t="s">
-        <v>140</v>
+      <c r="I79" s="6" t="s">
+        <v>139</v>
       </c>
       <c r="J79"/>
       <c r="K79"/>
-    </row>
-    <row r="80" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B80" s="40"/>
-      <c r="C80" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="D80" s="27" t="str">
+      <c r="L79"/>
+    </row>
+    <row r="80" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B80" s="37"/>
+      <c r="C80" s="24" t="s">
+        <v>147</v>
+      </c>
+      <c r="D80" s="25" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="E80" s="27" t="str">
+      <c r="E80" s="25" t="str">
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="F80" s="28" t="s">
-        <v>121</v>
-      </c>
-      <c r="G80" s="27" t="s">
+      <c r="F80" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="G80" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="H80" s="27" t="s">
-        <v>87</v>
-      </c>
-      <c r="I80" s="29" t="s">
-        <v>140</v>
+      <c r="H80" s="25" t="s">
+        <v>87</v>
+      </c>
+      <c r="I80" s="27" t="s">
+        <v>139</v>
       </c>
       <c r="J80"/>
       <c r="K80"/>
-    </row>
-    <row r="81" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B81" s="40"/>
-      <c r="C81" s="6" t="s">
-        <v>145</v>
+      <c r="L80"/>
+    </row>
+    <row r="81" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B81" s="37"/>
+      <c r="C81" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="D81" s="2" t="str">
         <f t="shared" si="2"/>
@@ -3241,100 +3624,163 @@
         <f t="shared" si="2"/>
         <v>-</v>
       </c>
-      <c r="F81" s="25" t="s">
-        <v>122</v>
+      <c r="F81" s="23" t="s">
+        <v>121</v>
       </c>
       <c r="G81" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H81" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="I81" s="7" t="str">
+        <v>140</v>
+      </c>
+      <c r="I81" s="6" t="str">
         <f t="shared" ref="I81" si="3">"-"</f>
         <v>-</v>
       </c>
       <c r="J81"/>
       <c r="K81"/>
-    </row>
-    <row r="82" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B82" s="40"/>
-      <c r="C82" s="30"/>
-      <c r="D82" s="31"/>
-      <c r="E82" s="31"/>
-      <c r="F82" s="31"/>
-      <c r="G82" s="31"/>
-      <c r="H82" s="31"/>
-      <c r="I82" s="32"/>
+      <c r="L81"/>
+    </row>
+    <row r="82" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B82" s="37"/>
+      <c r="C82" s="28"/>
+      <c r="D82" s="29"/>
+      <c r="E82" s="29"/>
+      <c r="F82" s="29"/>
+      <c r="G82" s="29"/>
+      <c r="H82" s="29"/>
+      <c r="I82" s="30"/>
       <c r="J82"/>
       <c r="K82"/>
-    </row>
-    <row r="83" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B83" s="40"/>
-      <c r="D83" s="15"/>
-      <c r="E83" s="15"/>
-      <c r="F83" s="15"/>
-      <c r="G83" s="15"/>
-      <c r="H83" s="15"/>
-      <c r="I83" s="16"/>
+      <c r="L82"/>
+    </row>
+    <row r="83" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B83" s="37"/>
+      <c r="D83" s="14"/>
+      <c r="E83" s="14"/>
+      <c r="F83" s="14"/>
+      <c r="G83" s="14"/>
+      <c r="H83" s="14"/>
+      <c r="I83" s="15"/>
       <c r="J83"/>
       <c r="K83"/>
-    </row>
-    <row r="84" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B84" s="46"/>
-      <c r="C84" s="26" t="s">
-        <v>144</v>
-      </c>
-      <c r="D84" s="27"/>
-      <c r="E84" s="27"/>
-      <c r="F84" s="27"/>
-      <c r="G84" s="27"/>
-      <c r="H84" s="27"/>
-      <c r="I84" s="29"/>
+      <c r="L83"/>
+    </row>
+    <row r="84" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B84" s="38"/>
+      <c r="C84" s="24" t="s">
+        <v>143</v>
+      </c>
+      <c r="D84" s="25"/>
+      <c r="E84" s="25"/>
+      <c r="F84" s="25"/>
+      <c r="G84" s="25"/>
+      <c r="H84" s="25"/>
+      <c r="I84" s="27"/>
       <c r="J84"/>
       <c r="K84"/>
-    </row>
-    <row r="85" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B85" s="40"/>
-      <c r="C85" s="26" t="s">
-        <v>146</v>
-      </c>
-      <c r="D85" s="27"/>
-      <c r="E85" s="27"/>
-      <c r="F85" s="27"/>
-      <c r="G85" s="27"/>
-      <c r="H85" s="27"/>
-      <c r="I85" s="29"/>
+      <c r="L84"/>
+    </row>
+    <row r="85" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B85" s="37"/>
+      <c r="C85" s="24" t="s">
+        <v>145</v>
+      </c>
+      <c r="D85" s="25"/>
+      <c r="E85" s="25"/>
+      <c r="F85" s="25"/>
+      <c r="G85" s="25"/>
+      <c r="H85" s="25"/>
+      <c r="I85" s="27"/>
       <c r="J85"/>
       <c r="K85"/>
-      <c r="L85" s="1"/>
-    </row>
-    <row r="86" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B86" s="41"/>
-      <c r="C86" s="33" t="s">
-        <v>147</v>
-      </c>
-      <c r="D86" s="34"/>
-      <c r="E86" s="34"/>
-      <c r="F86" s="34"/>
-      <c r="G86" s="34"/>
-      <c r="H86" s="34"/>
-      <c r="I86" s="35"/>
+      <c r="L85"/>
+      <c r="M85" s="1"/>
+    </row>
+    <row r="86" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B86" s="39"/>
+      <c r="C86" s="31" t="s">
+        <v>146</v>
+      </c>
+      <c r="D86" s="32"/>
+      <c r="E86" s="32"/>
+      <c r="F86" s="32"/>
+      <c r="G86" s="32"/>
+      <c r="H86" s="32"/>
+      <c r="I86" s="33"/>
       <c r="J86"/>
       <c r="K86"/>
-      <c r="L86" s="1"/>
-    </row>
-    <row r="87" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B87" s="24"/>
-    </row>
-    <row r="88" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B88" s="24"/>
-    </row>
-    <row r="89" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B89" s="24"/>
+      <c r="L86"/>
+      <c r="M86" s="1"/>
+    </row>
+    <row r="87" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B87" s="22"/>
+    </row>
+    <row r="88" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B88" s="22"/>
+    </row>
+    <row r="89" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B89" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="45">
+  <mergeCells count="73">
+    <mergeCell ref="L49:M49"/>
+    <mergeCell ref="L50:M50"/>
+    <mergeCell ref="L51:M51"/>
+    <mergeCell ref="L52:M52"/>
+    <mergeCell ref="K53:N53"/>
+    <mergeCell ref="L44:M44"/>
+    <mergeCell ref="L45:M45"/>
+    <mergeCell ref="L46:M46"/>
+    <mergeCell ref="L47:M47"/>
+    <mergeCell ref="L48:M48"/>
+    <mergeCell ref="L39:M39"/>
+    <mergeCell ref="L40:M40"/>
+    <mergeCell ref="L41:M41"/>
+    <mergeCell ref="L42:M42"/>
+    <mergeCell ref="L43:M43"/>
+    <mergeCell ref="L34:M34"/>
+    <mergeCell ref="L35:M35"/>
+    <mergeCell ref="L36:M36"/>
+    <mergeCell ref="L37:M37"/>
+    <mergeCell ref="L38:M38"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="K33:M33"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="K6:K7"/>
+    <mergeCell ref="K10:K26"/>
+    <mergeCell ref="D19:D22"/>
+    <mergeCell ref="E3:E6"/>
+    <mergeCell ref="D3:D6"/>
+    <mergeCell ref="D15:D18"/>
+    <mergeCell ref="D7:D10"/>
+    <mergeCell ref="D11:D14"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="C23:C27"/>
+    <mergeCell ref="C28:C32"/>
+    <mergeCell ref="C33:C37"/>
+    <mergeCell ref="C38:C42"/>
+    <mergeCell ref="E46:E48"/>
+    <mergeCell ref="D38:D42"/>
+    <mergeCell ref="D28:D32"/>
+    <mergeCell ref="D46:D48"/>
+    <mergeCell ref="B3:B22"/>
+    <mergeCell ref="C3:C6"/>
+    <mergeCell ref="C7:C10"/>
+    <mergeCell ref="C11:C14"/>
+    <mergeCell ref="C15:C18"/>
+    <mergeCell ref="C19:C22"/>
+    <mergeCell ref="C49:C51"/>
+    <mergeCell ref="B43:B51"/>
+    <mergeCell ref="D43:D45"/>
+    <mergeCell ref="C43:C45"/>
+    <mergeCell ref="C46:C48"/>
     <mergeCell ref="B68:B86"/>
     <mergeCell ref="E7:E10"/>
     <mergeCell ref="E11:E14"/>
@@ -3351,35 +3797,6 @@
     <mergeCell ref="B23:B42"/>
     <mergeCell ref="B52:B67"/>
     <mergeCell ref="D49:D51"/>
-    <mergeCell ref="C49:C51"/>
-    <mergeCell ref="B43:B51"/>
-    <mergeCell ref="D43:D45"/>
-    <mergeCell ref="C43:C45"/>
-    <mergeCell ref="C46:C48"/>
-    <mergeCell ref="B3:B22"/>
-    <mergeCell ref="C3:C6"/>
-    <mergeCell ref="C7:C10"/>
-    <mergeCell ref="C11:C14"/>
-    <mergeCell ref="C15:C18"/>
-    <mergeCell ref="C19:C22"/>
-    <mergeCell ref="C23:C27"/>
-    <mergeCell ref="C28:C32"/>
-    <mergeCell ref="C33:C37"/>
-    <mergeCell ref="C38:C42"/>
-    <mergeCell ref="E46:E48"/>
-    <mergeCell ref="D38:D42"/>
-    <mergeCell ref="D28:D32"/>
-    <mergeCell ref="D46:D48"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="K6:K7"/>
-    <mergeCell ref="K10:K26"/>
-    <mergeCell ref="D19:D22"/>
-    <mergeCell ref="E3:E6"/>
-    <mergeCell ref="D3:D6"/>
-    <mergeCell ref="D15:D18"/>
-    <mergeCell ref="D7:D10"/>
-    <mergeCell ref="D11:D14"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>